<commit_message>
Remove obsolete scripts related to Puno network configuration and server setup, including generar_puno_direccionamiento.py, generar_sede_principal_wan.py, generar_sede_vlsm_comun.py, generar_tabla_subredes.py, and servidores-gig.MD. These files are no longer needed for the current project structure and functionality.
</commit_message>
<xml_diff>
--- a/excel-final/Esquema de Direccionamiento IP.xlsx
+++ b/excel-final/Esquema de Direccionamiento IP.xlsx
@@ -17,7 +17,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="728" uniqueCount="378">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="734" uniqueCount="384">
   <si>
     <t>Caso Estudio:</t>
   </si>
@@ -508,6 +508,9 @@
     <t>Mascara de Subred</t>
   </si>
   <si>
+    <t>Direccion de Broadcast</t>
+  </si>
+  <si>
     <t>Ventas</t>
   </si>
   <si>
@@ -652,171 +655,180 @@
     <t>10.192.42.159</t>
   </si>
   <si>
+    <t>Nativa</t>
+  </si>
+  <si>
+    <t>VLNAT</t>
+  </si>
+  <si>
+    <t>10.192.42.160</t>
+  </si>
+  <si>
+    <t>10.192.42.161</t>
+  </si>
+  <si>
+    <t>10.192.42.190</t>
+  </si>
+  <si>
+    <t>10.192.42.191</t>
+  </si>
+  <si>
+    <t>Servidores</t>
+  </si>
+  <si>
+    <t>VLSER</t>
+  </si>
+  <si>
+    <t>/28</t>
+  </si>
+  <si>
+    <t>255.255.255.240</t>
+  </si>
+  <si>
+    <t>10.192.42.192</t>
+  </si>
+  <si>
+    <t>10.192.42.193</t>
+  </si>
+  <si>
+    <t>10.192.42.206</t>
+  </si>
+  <si>
+    <t>10.192.42.207</t>
+  </si>
+  <si>
+    <t>Nota:</t>
+  </si>
+  <si>
+    <t>Nativa se calculo con 15 equipos actuales asumidos para gestion; ajustar si tu Packet Tracer usa otra cantidad. XYZW queda reservado.</t>
+  </si>
+  <si>
+    <t>Validacion:</t>
+  </si>
+  <si>
+    <t>Todas las VLAN quedan dentro de 10.192.40.0/22 y no se solapan.</t>
+  </si>
+  <si>
+    <t>Yeremi Tanner Villavicencio Rios</t>
+  </si>
+  <si>
+    <t>10.192.44.0/22</t>
+  </si>
+  <si>
+    <t>10.192.44.126</t>
+  </si>
+  <si>
+    <t>10.192.44.127</t>
+  </si>
+  <si>
+    <t>10.192.44.128</t>
+  </si>
+  <si>
+    <t>10.192.44.129</t>
+  </si>
+  <si>
+    <t>10.192.44.190</t>
+  </si>
+  <si>
+    <t>10.192.44.191</t>
+  </si>
+  <si>
+    <t>10.192.44.192</t>
+  </si>
+  <si>
+    <t>10.192.44.193</t>
+  </si>
+  <si>
+    <t>10.192.44.222</t>
+  </si>
+  <si>
+    <t>10.192.44.223</t>
+  </si>
+  <si>
+    <t>10.192.44.224</t>
+  </si>
+  <si>
+    <t>10.192.44.225</t>
+  </si>
+  <si>
+    <t>10.192.44.238</t>
+  </si>
+  <si>
+    <t>10.192.44.239</t>
+  </si>
+  <si>
+    <t>10.192.44.240</t>
+  </si>
+  <si>
+    <t>10.192.44.241</t>
+  </si>
+  <si>
+    <t>10.192.44.254</t>
+  </si>
+  <si>
+    <t>10.192.44.255</t>
+  </si>
+  <si>
+    <t>10.192.45.0</t>
+  </si>
+  <si>
+    <t>10.192.45.1</t>
+  </si>
+  <si>
+    <t>10.192.45.14</t>
+  </si>
+  <si>
+    <t>10.192.45.15</t>
+  </si>
+  <si>
+    <t>10.192.45.16</t>
+  </si>
+  <si>
+    <t>10.192.45.17</t>
+  </si>
+  <si>
+    <t>10.192.45.30</t>
+  </si>
+  <si>
+    <t>10.192.45.31</t>
+  </si>
+  <si>
     <t>Nativa/Gestion</t>
   </si>
   <si>
-    <t>VLNAT</t>
-  </si>
-  <si>
-    <t>10.192.42.160</t>
-  </si>
-  <si>
-    <t>10.192.42.161</t>
-  </si>
-  <si>
-    <t>10.192.42.190</t>
-  </si>
-  <si>
-    <t>10.192.42.191</t>
-  </si>
-  <si>
-    <t>Servidores</t>
-  </si>
-  <si>
-    <t>VLSER</t>
-  </si>
-  <si>
-    <t>/28</t>
-  </si>
-  <si>
-    <t>255.255.255.240</t>
-  </si>
-  <si>
-    <t>10.192.42.192</t>
-  </si>
-  <si>
-    <t>10.192.42.193</t>
-  </si>
-  <si>
-    <t>10.192.42.206</t>
-  </si>
-  <si>
-    <t>10.192.42.207</t>
+    <t>/29</t>
+  </si>
+  <si>
+    <t>255.255.255.248</t>
+  </si>
+  <si>
+    <t>10.192.45.32</t>
+  </si>
+  <si>
+    <t>10.192.45.33</t>
+  </si>
+  <si>
+    <t>10.192.45.38</t>
+  </si>
+  <si>
+    <t>10.192.45.39</t>
+  </si>
+  <si>
+    <t>10.192.45.40</t>
+  </si>
+  <si>
+    <t>10.192.45.41</t>
+  </si>
+  <si>
+    <t>10.192.45.46</t>
+  </si>
+  <si>
+    <t>10.192.45.47</t>
   </si>
   <si>
     <t>Total Host</t>
   </si>
   <si>
-    <t>Yeremi Tanner Villavicencio Rios</t>
-  </si>
-  <si>
-    <t>10.192.44.0/22</t>
-  </si>
-  <si>
-    <t>Direccion de Broadcast</t>
-  </si>
-  <si>
-    <t>10.192.44.126</t>
-  </si>
-  <si>
-    <t>10.192.44.127</t>
-  </si>
-  <si>
-    <t>10.192.44.128</t>
-  </si>
-  <si>
-    <t>10.192.44.129</t>
-  </si>
-  <si>
-    <t>10.192.44.190</t>
-  </si>
-  <si>
-    <t>10.192.44.191</t>
-  </si>
-  <si>
-    <t>10.192.44.192</t>
-  </si>
-  <si>
-    <t>10.192.44.193</t>
-  </si>
-  <si>
-    <t>10.192.44.222</t>
-  </si>
-  <si>
-    <t>10.192.44.223</t>
-  </si>
-  <si>
-    <t>10.192.44.224</t>
-  </si>
-  <si>
-    <t>10.192.44.225</t>
-  </si>
-  <si>
-    <t>10.192.44.238</t>
-  </si>
-  <si>
-    <t>10.192.44.239</t>
-  </si>
-  <si>
-    <t>10.192.44.240</t>
-  </si>
-  <si>
-    <t>10.192.44.241</t>
-  </si>
-  <si>
-    <t>10.192.44.254</t>
-  </si>
-  <si>
-    <t>10.192.44.255</t>
-  </si>
-  <si>
-    <t>10.192.45.0</t>
-  </si>
-  <si>
-    <t>10.192.45.1</t>
-  </si>
-  <si>
-    <t>10.192.45.14</t>
-  </si>
-  <si>
-    <t>10.192.45.15</t>
-  </si>
-  <si>
-    <t>10.192.45.16</t>
-  </si>
-  <si>
-    <t>10.192.45.17</t>
-  </si>
-  <si>
-    <t>10.192.45.30</t>
-  </si>
-  <si>
-    <t>10.192.45.31</t>
-  </si>
-  <si>
-    <t>/29</t>
-  </si>
-  <si>
-    <t>255.255.255.248</t>
-  </si>
-  <si>
-    <t>10.192.45.32</t>
-  </si>
-  <si>
-    <t>10.192.45.33</t>
-  </si>
-  <si>
-    <t>10.192.45.38</t>
-  </si>
-  <si>
-    <t>10.192.45.39</t>
-  </si>
-  <si>
-    <t>10.192.45.40</t>
-  </si>
-  <si>
-    <t>10.192.45.41</t>
-  </si>
-  <si>
-    <t>10.192.45.46</t>
-  </si>
-  <si>
-    <t>10.192.45.47</t>
-  </si>
-  <si>
-    <t>Validacion:</t>
-  </si>
-  <si>
     <t>Todas las VLAN quedan dentro de 10.192.44.0/22 y no se solapan.</t>
   </si>
   <si>
@@ -937,6 +949,18 @@
     <t>10.192.52.0/22</t>
   </si>
   <si>
+    <t>10.192.52.30</t>
+  </si>
+  <si>
+    <t>10.192.52.31</t>
+  </si>
+  <si>
+    <t>10.192.52.32</t>
+  </si>
+  <si>
+    <t>10.192.52.33</t>
+  </si>
+  <si>
     <t>10.192.52.62</t>
   </si>
   <si>
@@ -1021,18 +1045,6 @@
     <t>10.192.52.177</t>
   </si>
   <si>
-    <t>10.192.52.182</t>
-  </si>
-  <si>
-    <t>10.192.52.183</t>
-  </si>
-  <si>
-    <t>10.192.52.184</t>
-  </si>
-  <si>
-    <t>10.192.52.185</t>
-  </si>
-  <si>
     <t>10.192.52.190</t>
   </si>
   <si>
@@ -1151,6 +1163,12 @@
   </si>
   <si>
     <t>Todas las VLAN quedan dentro de 10.192.56.0/22 y no se solapan.</t>
+  </si>
+  <si>
+    <t>10.192.56.114</t>
+  </si>
+  <si>
+    <t>10.192.56.115</t>
   </si>
 </sst>
 </file>
@@ -1195,7 +1213,7 @@
     <font>
       <b/>
       <sz val="11.0"/>
-      <color rgb="FF000000"/>
+      <color rgb="FFFFFFFF"/>
       <name val="Calibri"/>
     </font>
     <font>
@@ -1206,7 +1224,7 @@
     <font>
       <b/>
       <sz val="11.0"/>
-      <color rgb="FFFFFFFF"/>
+      <color rgb="FF000000"/>
       <name val="Calibri"/>
     </font>
   </fonts>
@@ -1286,7 +1304,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="35">
+  <cellXfs count="37">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -1351,33 +1369,28 @@
     <xf borderId="2" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0" vertical="bottom"/>
     </xf>
-    <xf borderId="1" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0" shrinkToFit="0" wrapText="1"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyFont="1"/>
-    <xf borderId="1" fillId="0" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
-    </xf>
-    <xf borderId="2" fillId="0" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
-    </xf>
-    <xf borderId="4" fillId="0" fontId="6" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
-    <xf borderId="0" fillId="0" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment shrinkToFit="0" vertical="bottom" wrapText="0"/>
-    </xf>
-    <xf borderId="1" fillId="0" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
-    </xf>
-    <xf borderId="1" fillId="4" fontId="9" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="1" fillId="4" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
     <xf borderId="1" fillId="0" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0" shrinkToFit="0" wrapText="0"/>
     </xf>
-    <xf borderId="1" fillId="0" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="1" fillId="0" fontId="9" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
+    </xf>
+    <xf borderId="1" fillId="0" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
+    </xf>
+    <xf borderId="4" fillId="0" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
+    </xf>
+    <xf borderId="3" fillId="0" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment shrinkToFit="0" vertical="bottom" wrapText="0"/>
+    </xf>
+    <xf borderId="1" fillId="0" fontId="9" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="right" readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
@@ -1385,6 +1398,19 @@
     </xf>
     <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf borderId="1" fillId="4" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
+    </xf>
+    <xf borderId="1" fillId="0" fontId="8" numFmtId="1" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
+      <alignment horizontal="center" readingOrder="0" shrinkToFit="0" wrapText="0"/>
+    </xf>
+    <xf borderId="2" fillId="0" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
+    </xf>
+    <xf borderId="4" fillId="0" fontId="6" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
+    <xf borderId="1" fillId="4" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0" shrinkToFit="0" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -2664,7 +2690,7 @@
         <v>162</v>
       </c>
       <c r="J6" s="22" t="s">
-        <v>12</v>
+        <v>127</v>
       </c>
       <c r="K6" s="22" t="s">
         <v>15</v>
@@ -2673,389 +2699,392 @@
         <v>16</v>
       </c>
       <c r="M6" s="22" t="s">
-        <v>17</v>
+        <v>163</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="2" t="s">
-        <v>163</v>
-      </c>
-      <c r="B7" s="2">
+      <c r="A7" s="23" t="s">
+        <v>164</v>
+      </c>
+      <c r="B7" s="23">
         <v>198.0</v>
       </c>
-      <c r="C7" s="2">
+      <c r="C7" s="23">
         <v>248.0</v>
       </c>
-      <c r="D7" s="2" t="s">
-        <v>164</v>
-      </c>
-      <c r="E7" s="2">
+      <c r="D7" s="23" t="s">
+        <v>165</v>
+      </c>
+      <c r="E7" s="23">
         <v>10.0</v>
       </c>
-      <c r="F7" s="2">
+      <c r="F7" s="23">
         <v>8.0</v>
       </c>
-      <c r="G7" s="2">
+      <c r="G7" s="23">
         <v>254.0</v>
       </c>
-      <c r="H7" s="2" t="s">
-        <v>165</v>
-      </c>
-      <c r="I7" s="2" t="s">
+      <c r="H7" s="23" t="s">
         <v>166</v>
       </c>
-      <c r="J7" s="2" t="s">
+      <c r="I7" s="23" t="s">
+        <v>167</v>
+      </c>
+      <c r="J7" s="23" t="s">
         <v>94</v>
       </c>
-      <c r="K7" s="2" t="s">
+      <c r="K7" s="23" t="s">
         <v>95</v>
       </c>
-      <c r="L7" s="2" t="s">
-        <v>167</v>
-      </c>
-      <c r="M7" s="2" t="s">
+      <c r="L7" s="23" t="s">
         <v>168</v>
       </c>
+      <c r="M7" s="23" t="s">
+        <v>169</v>
+      </c>
     </row>
     <row r="8">
-      <c r="A8" s="2" t="s">
-        <v>169</v>
-      </c>
-      <c r="B8" s="2">
+      <c r="A8" s="23" t="s">
+        <v>170</v>
+      </c>
+      <c r="B8" s="23">
         <v>100.0</v>
       </c>
-      <c r="C8" s="2">
+      <c r="C8" s="23">
         <v>125.0</v>
       </c>
-      <c r="D8" s="2" t="s">
-        <v>170</v>
-      </c>
-      <c r="E8" s="2">
+      <c r="D8" s="23" t="s">
+        <v>171</v>
+      </c>
+      <c r="E8" s="23">
         <v>11.0</v>
       </c>
-      <c r="F8" s="2">
+      <c r="F8" s="23">
         <v>7.0</v>
       </c>
-      <c r="G8" s="2">
+      <c r="G8" s="23">
         <v>126.0</v>
       </c>
-      <c r="H8" s="2" t="s">
-        <v>171</v>
-      </c>
-      <c r="I8" s="2" t="s">
+      <c r="H8" s="23" t="s">
         <v>172</v>
       </c>
-      <c r="J8" s="2" t="s">
+      <c r="I8" s="23" t="s">
         <v>173</v>
       </c>
-      <c r="K8" s="2" t="s">
+      <c r="J8" s="23" t="s">
         <v>174</v>
       </c>
-      <c r="L8" s="2" t="s">
+      <c r="K8" s="23" t="s">
         <v>175</v>
       </c>
-      <c r="M8" s="2" t="s">
+      <c r="L8" s="23" t="s">
         <v>176</v>
       </c>
+      <c r="M8" s="23" t="s">
+        <v>177</v>
+      </c>
     </row>
     <row r="9">
-      <c r="A9" s="2" t="s">
-        <v>177</v>
-      </c>
-      <c r="B9" s="2">
+      <c r="A9" s="23" t="s">
+        <v>178</v>
+      </c>
+      <c r="B9" s="23">
         <v>41.0</v>
       </c>
-      <c r="C9" s="2">
+      <c r="C9" s="23">
         <v>52.0</v>
       </c>
-      <c r="D9" s="2" t="s">
-        <v>178</v>
-      </c>
-      <c r="E9" s="2">
+      <c r="D9" s="23" t="s">
+        <v>179</v>
+      </c>
+      <c r="E9" s="23">
         <v>12.0</v>
       </c>
-      <c r="F9" s="2">
+      <c r="F9" s="23">
         <v>6.0</v>
       </c>
-      <c r="G9" s="2">
+      <c r="G9" s="23">
         <v>62.0</v>
       </c>
-      <c r="H9" s="2" t="s">
-        <v>179</v>
-      </c>
-      <c r="I9" s="2" t="s">
+      <c r="H9" s="23" t="s">
         <v>180</v>
       </c>
-      <c r="J9" s="2" t="s">
+      <c r="I9" s="23" t="s">
         <v>181</v>
       </c>
-      <c r="K9" s="2" t="s">
+      <c r="J9" s="23" t="s">
         <v>182</v>
       </c>
-      <c r="L9" s="2" t="s">
+      <c r="K9" s="23" t="s">
         <v>183</v>
       </c>
-      <c r="M9" s="2" t="s">
+      <c r="L9" s="23" t="s">
         <v>184</v>
       </c>
+      <c r="M9" s="23" t="s">
+        <v>185</v>
+      </c>
     </row>
     <row r="10">
-      <c r="A10" s="2" t="s">
-        <v>185</v>
-      </c>
-      <c r="B10" s="2">
+      <c r="A10" s="23" t="s">
+        <v>186</v>
+      </c>
+      <c r="B10" s="23">
         <v>31.0</v>
       </c>
-      <c r="C10" s="2">
+      <c r="C10" s="23">
         <v>39.0</v>
       </c>
-      <c r="D10" s="2" t="s">
-        <v>186</v>
-      </c>
-      <c r="E10" s="2">
+      <c r="D10" s="23" t="s">
+        <v>187</v>
+      </c>
+      <c r="E10" s="23">
         <v>13.0</v>
       </c>
-      <c r="F10" s="2">
+      <c r="F10" s="23">
         <v>6.0</v>
       </c>
-      <c r="G10" s="2">
+      <c r="G10" s="23">
         <v>62.0</v>
       </c>
-      <c r="H10" s="2" t="s">
-        <v>179</v>
-      </c>
-      <c r="I10" s="2" t="s">
+      <c r="H10" s="23" t="s">
         <v>180</v>
       </c>
-      <c r="J10" s="2" t="s">
-        <v>187</v>
-      </c>
-      <c r="K10" s="2" t="s">
+      <c r="I10" s="23" t="s">
+        <v>181</v>
+      </c>
+      <c r="J10" s="23" t="s">
         <v>188</v>
       </c>
-      <c r="L10" s="2" t="s">
+      <c r="K10" s="23" t="s">
         <v>189</v>
       </c>
-      <c r="M10" s="2" t="s">
+      <c r="L10" s="23" t="s">
         <v>190</v>
       </c>
+      <c r="M10" s="23" t="s">
+        <v>191</v>
+      </c>
     </row>
     <row r="11">
-      <c r="A11" s="2" t="s">
-        <v>191</v>
-      </c>
-      <c r="B11" s="2">
+      <c r="A11" s="23" t="s">
+        <v>192</v>
+      </c>
+      <c r="B11" s="23">
         <v>29.0</v>
       </c>
-      <c r="C11" s="2">
+      <c r="C11" s="23">
         <v>37.0</v>
       </c>
-      <c r="D11" s="2" t="s">
-        <v>192</v>
-      </c>
-      <c r="E11" s="2">
+      <c r="D11" s="23" t="s">
+        <v>193</v>
+      </c>
+      <c r="E11" s="23">
         <v>14.0</v>
       </c>
-      <c r="F11" s="2">
+      <c r="F11" s="23">
         <v>6.0</v>
       </c>
-      <c r="G11" s="2">
+      <c r="G11" s="23">
         <v>62.0</v>
       </c>
-      <c r="H11" s="2" t="s">
-        <v>179</v>
-      </c>
-      <c r="I11" s="2" t="s">
+      <c r="H11" s="23" t="s">
         <v>180</v>
       </c>
-      <c r="J11" s="2" t="s">
-        <v>193</v>
-      </c>
-      <c r="K11" s="2" t="s">
+      <c r="I11" s="23" t="s">
+        <v>181</v>
+      </c>
+      <c r="J11" s="23" t="s">
         <v>194</v>
       </c>
-      <c r="L11" s="2" t="s">
+      <c r="K11" s="23" t="s">
         <v>195</v>
       </c>
-      <c r="M11" s="2" t="s">
+      <c r="L11" s="23" t="s">
         <v>196</v>
       </c>
+      <c r="M11" s="23" t="s">
+        <v>197</v>
+      </c>
     </row>
     <row r="12">
-      <c r="A12" s="2" t="s">
-        <v>197</v>
-      </c>
-      <c r="B12" s="2">
+      <c r="A12" s="23" t="s">
+        <v>198</v>
+      </c>
+      <c r="B12" s="23">
         <v>25.0</v>
       </c>
-      <c r="C12" s="2">
+      <c r="C12" s="23">
         <v>32.0</v>
       </c>
-      <c r="D12" s="2" t="s">
-        <v>198</v>
-      </c>
-      <c r="E12" s="2">
+      <c r="D12" s="23" t="s">
+        <v>199</v>
+      </c>
+      <c r="E12" s="23">
         <v>15.0</v>
       </c>
-      <c r="F12" s="2">
+      <c r="F12" s="23">
         <v>6.0</v>
       </c>
-      <c r="G12" s="2">
+      <c r="G12" s="23">
         <v>62.0</v>
       </c>
-      <c r="H12" s="2" t="s">
-        <v>179</v>
-      </c>
-      <c r="I12" s="2" t="s">
+      <c r="H12" s="23" t="s">
         <v>180</v>
       </c>
-      <c r="J12" s="2" t="s">
-        <v>199</v>
-      </c>
-      <c r="K12" s="2" t="s">
+      <c r="I12" s="23" t="s">
+        <v>181</v>
+      </c>
+      <c r="J12" s="23" t="s">
         <v>200</v>
       </c>
-      <c r="L12" s="2" t="s">
+      <c r="K12" s="23" t="s">
         <v>201</v>
       </c>
-      <c r="M12" s="2" t="s">
+      <c r="L12" s="23" t="s">
         <v>202</v>
       </c>
+      <c r="M12" s="23" t="s">
+        <v>203</v>
+      </c>
     </row>
     <row r="13">
-      <c r="A13" s="2" t="s">
-        <v>203</v>
-      </c>
-      <c r="B13" s="2">
+      <c r="A13" s="23" t="s">
+        <v>204</v>
+      </c>
+      <c r="B13" s="23">
         <v>18.0</v>
       </c>
-      <c r="C13" s="2">
+      <c r="C13" s="23">
         <v>23.0</v>
       </c>
-      <c r="D13" s="2" t="s">
-        <v>204</v>
-      </c>
-      <c r="E13" s="2">
+      <c r="D13" s="23" t="s">
+        <v>205</v>
+      </c>
+      <c r="E13" s="23">
         <v>16.0</v>
       </c>
-      <c r="F13" s="2">
+      <c r="F13" s="23">
         <v>5.0</v>
       </c>
-      <c r="G13" s="2">
+      <c r="G13" s="23">
         <v>30.0</v>
       </c>
-      <c r="H13" s="2" t="s">
-        <v>205</v>
-      </c>
-      <c r="I13" s="2" t="s">
+      <c r="H13" s="23" t="s">
         <v>206</v>
       </c>
-      <c r="J13" s="2" t="s">
+      <c r="I13" s="23" t="s">
         <v>207</v>
       </c>
-      <c r="K13" s="2" t="s">
+      <c r="J13" s="23" t="s">
         <v>208</v>
       </c>
-      <c r="L13" s="2" t="s">
+      <c r="K13" s="23" t="s">
         <v>209</v>
       </c>
-      <c r="M13" s="2" t="s">
+      <c r="L13" s="23" t="s">
         <v>210</v>
       </c>
+      <c r="M13" s="23" t="s">
+        <v>211</v>
+      </c>
     </row>
     <row r="14">
-      <c r="A14" s="2" t="s">
-        <v>211</v>
-      </c>
-      <c r="B14" s="2">
+      <c r="A14" s="23" t="s">
+        <v>212</v>
+      </c>
+      <c r="B14" s="23">
         <v>15.0</v>
       </c>
-      <c r="C14" s="2">
+      <c r="C14" s="23">
         <v>19.0</v>
       </c>
-      <c r="D14" s="2" t="s">
-        <v>212</v>
-      </c>
-      <c r="E14" s="2">
+      <c r="D14" s="23" t="s">
+        <v>213</v>
+      </c>
+      <c r="E14" s="23">
         <v>99.0</v>
       </c>
-      <c r="F14" s="2">
+      <c r="F14" s="23">
         <v>5.0</v>
       </c>
-      <c r="G14" s="2">
+      <c r="G14" s="23">
         <v>30.0</v>
       </c>
-      <c r="H14" s="2" t="s">
-        <v>205</v>
-      </c>
-      <c r="I14" s="2" t="s">
+      <c r="H14" s="23" t="s">
         <v>206</v>
       </c>
-      <c r="J14" s="2" t="s">
-        <v>213</v>
-      </c>
-      <c r="K14" s="2" t="s">
+      <c r="I14" s="23" t="s">
+        <v>207</v>
+      </c>
+      <c r="J14" s="23" t="s">
         <v>214</v>
       </c>
-      <c r="L14" s="2" t="s">
+      <c r="K14" s="23" t="s">
         <v>215</v>
       </c>
-      <c r="M14" s="2" t="s">
+      <c r="L14" s="23" t="s">
         <v>216</v>
       </c>
+      <c r="M14" s="23" t="s">
+        <v>217</v>
+      </c>
     </row>
     <row r="15">
-      <c r="A15" s="2" t="s">
-        <v>217</v>
-      </c>
-      <c r="B15" s="2">
+      <c r="A15" s="23" t="s">
+        <v>218</v>
+      </c>
+      <c r="B15" s="23">
         <v>10.0</v>
       </c>
-      <c r="C15" s="2">
+      <c r="C15" s="23">
         <v>13.0</v>
       </c>
-      <c r="D15" s="2" t="s">
-        <v>218</v>
-      </c>
-      <c r="E15" s="2">
+      <c r="D15" s="23" t="s">
+        <v>219</v>
+      </c>
+      <c r="E15" s="23">
         <v>17.0</v>
       </c>
-      <c r="F15" s="2">
+      <c r="F15" s="23">
         <v>4.0</v>
       </c>
-      <c r="G15" s="2">
+      <c r="G15" s="23">
         <v>14.0</v>
       </c>
-      <c r="H15" s="2" t="s">
-        <v>219</v>
-      </c>
-      <c r="I15" s="2" t="s">
+      <c r="H15" s="23" t="s">
         <v>220</v>
       </c>
-      <c r="J15" s="2" t="s">
+      <c r="I15" s="23" t="s">
         <v>221</v>
       </c>
-      <c r="K15" s="2" t="s">
+      <c r="J15" s="23" t="s">
         <v>222</v>
       </c>
-      <c r="L15" s="2" t="s">
+      <c r="K15" s="23" t="s">
         <v>223</v>
       </c>
-      <c r="M15" s="2" t="s">
+      <c r="L15" s="23" t="s">
         <v>224</v>
       </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="23" t="s">
+      <c r="M15" s="23" t="s">
         <v>225</v>
       </c>
-      <c r="B16" s="24">
-        <f t="shared" ref="B16:C16" si="1">SUM(B7:B15)</f>
-        <v>467</v>
-      </c>
-      <c r="C16" s="24">
-        <f t="shared" si="1"/>
-        <v>588</v>
+    </row>
+    <row r="18">
+      <c r="A18" s="24" t="s">
+        <v>226</v>
+      </c>
+      <c r="B18" s="25" t="s">
+        <v>227</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="24" t="s">
+        <v>228</v>
+      </c>
+      <c r="B19" s="25" t="s">
+        <v>229</v>
       </c>
     </row>
   </sheetData>
@@ -3077,7 +3106,7 @@
   <cols>
     <col customWidth="1" min="1" max="1" width="33.0"/>
     <col customWidth="1" min="2" max="2" width="25.88"/>
-    <col customWidth="1" min="3" max="3" width="51.63"/>
+    <col customWidth="1" min="3" max="3" width="41.75"/>
     <col customWidth="1" min="4" max="4" width="23.25"/>
     <col customWidth="1" min="5" max="5" width="13.13"/>
     <col customWidth="1" min="7" max="7" width="18.25"/>
@@ -3090,14 +3119,14 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="25" t="s">
+      <c r="A1" s="24" t="s">
         <v>150</v>
       </c>
-      <c r="B1" s="26" t="s">
-        <v>226</v>
-      </c>
-      <c r="C1" s="27"/>
-      <c r="D1" s="18"/>
+      <c r="B1" s="25" t="s">
+        <v>230</v>
+      </c>
+      <c r="C1" s="26"/>
+      <c r="D1" s="27"/>
       <c r="E1" s="28"/>
       <c r="F1" s="28"/>
       <c r="G1" s="28"/>
@@ -3109,10 +3138,10 @@
       <c r="M1" s="28"/>
     </row>
     <row r="2">
-      <c r="A2" s="25" t="s">
+      <c r="A2" s="24" t="s">
         <v>77</v>
       </c>
-      <c r="B2" s="29" t="s">
+      <c r="B2" s="25" t="s">
         <v>104</v>
       </c>
       <c r="C2" s="28"/>
@@ -3128,11 +3157,11 @@
       <c r="M2" s="28"/>
     </row>
     <row r="3">
-      <c r="A3" s="25" t="s">
+      <c r="A3" s="24" t="s">
         <v>79</v>
       </c>
-      <c r="B3" s="29" t="s">
-        <v>227</v>
+      <c r="B3" s="25" t="s">
+        <v>231</v>
       </c>
       <c r="C3" s="28"/>
       <c r="D3" s="28"/>
@@ -3177,430 +3206,430 @@
       <c r="M5" s="28"/>
     </row>
     <row r="6">
-      <c r="A6" s="30" t="s">
+      <c r="A6" s="22" t="s">
         <v>155</v>
       </c>
-      <c r="B6" s="30" t="s">
+      <c r="B6" s="22" t="s">
         <v>156</v>
       </c>
-      <c r="C6" s="30" t="s">
+      <c r="C6" s="22" t="s">
         <v>157</v>
       </c>
-      <c r="D6" s="30" t="s">
+      <c r="D6" s="22" t="s">
         <v>158</v>
       </c>
-      <c r="E6" s="30" t="s">
+      <c r="E6" s="22" t="s">
         <v>159</v>
       </c>
-      <c r="F6" s="30" t="s">
+      <c r="F6" s="22" t="s">
         <v>160</v>
       </c>
-      <c r="G6" s="30" t="s">
+      <c r="G6" s="22" t="s">
         <v>161</v>
       </c>
-      <c r="H6" s="30" t="s">
+      <c r="H6" s="22" t="s">
         <v>14</v>
       </c>
-      <c r="I6" s="30" t="s">
+      <c r="I6" s="22" t="s">
         <v>162</v>
       </c>
-      <c r="J6" s="30" t="s">
+      <c r="J6" s="22" t="s">
         <v>127</v>
       </c>
-      <c r="K6" s="30" t="s">
+      <c r="K6" s="22" t="s">
         <v>15</v>
       </c>
-      <c r="L6" s="30" t="s">
+      <c r="L6" s="22" t="s">
         <v>16</v>
       </c>
-      <c r="M6" s="30" t="s">
-        <v>228</v>
+      <c r="M6" s="22" t="s">
+        <v>163</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="31" t="s">
-        <v>163</v>
-      </c>
-      <c r="B7" s="31">
+      <c r="A7" s="23" t="s">
+        <v>164</v>
+      </c>
+      <c r="B7" s="23">
         <v>70.0</v>
       </c>
-      <c r="C7" s="31">
+      <c r="C7" s="23">
         <v>88.0</v>
       </c>
-      <c r="D7" s="31" t="s">
-        <v>164</v>
-      </c>
-      <c r="E7" s="31">
+      <c r="D7" s="23" t="s">
+        <v>165</v>
+      </c>
+      <c r="E7" s="23">
         <v>30.0</v>
       </c>
-      <c r="F7" s="31">
+      <c r="F7" s="23">
         <v>7.0</v>
       </c>
-      <c r="G7" s="31">
+      <c r="G7" s="23">
         <v>126.0</v>
       </c>
-      <c r="H7" s="31" t="s">
+      <c r="H7" s="23" t="s">
+        <v>172</v>
+      </c>
+      <c r="I7" s="23" t="s">
+        <v>173</v>
+      </c>
+      <c r="J7" s="23" t="s">
+        <v>100</v>
+      </c>
+      <c r="K7" s="23" t="s">
+        <v>101</v>
+      </c>
+      <c r="L7" s="23" t="s">
+        <v>232</v>
+      </c>
+      <c r="M7" s="23" t="s">
+        <v>233</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="23" t="s">
+        <v>170</v>
+      </c>
+      <c r="B8" s="23">
+        <v>35.0</v>
+      </c>
+      <c r="C8" s="23">
+        <v>44.0</v>
+      </c>
+      <c r="D8" s="23" t="s">
         <v>171</v>
       </c>
-      <c r="I7" s="31" t="s">
-        <v>172</v>
-      </c>
-      <c r="J7" s="31" t="s">
-        <v>100</v>
-      </c>
-      <c r="K7" s="31" t="s">
-        <v>101</v>
-      </c>
-      <c r="L7" s="31" t="s">
-        <v>229</v>
-      </c>
-      <c r="M7" s="31" t="s">
-        <v>230</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="31" t="s">
-        <v>169</v>
-      </c>
-      <c r="B8" s="31">
+      <c r="E8" s="23">
+        <v>31.0</v>
+      </c>
+      <c r="F8" s="23">
+        <v>6.0</v>
+      </c>
+      <c r="G8" s="23">
+        <v>62.0</v>
+      </c>
+      <c r="H8" s="23" t="s">
+        <v>180</v>
+      </c>
+      <c r="I8" s="23" t="s">
+        <v>181</v>
+      </c>
+      <c r="J8" s="23" t="s">
+        <v>234</v>
+      </c>
+      <c r="K8" s="23" t="s">
+        <v>235</v>
+      </c>
+      <c r="L8" s="23" t="s">
+        <v>236</v>
+      </c>
+      <c r="M8" s="23" t="s">
+        <v>237</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="23" t="s">
+        <v>178</v>
+      </c>
+      <c r="B9" s="23">
+        <v>15.0</v>
+      </c>
+      <c r="C9" s="23">
+        <v>19.0</v>
+      </c>
+      <c r="D9" s="23" t="s">
+        <v>179</v>
+      </c>
+      <c r="E9" s="23">
+        <v>32.0</v>
+      </c>
+      <c r="F9" s="23">
+        <v>5.0</v>
+      </c>
+      <c r="G9" s="23">
+        <v>30.0</v>
+      </c>
+      <c r="H9" s="23" t="s">
+        <v>206</v>
+      </c>
+      <c r="I9" s="23" t="s">
+        <v>207</v>
+      </c>
+      <c r="J9" s="23" t="s">
+        <v>238</v>
+      </c>
+      <c r="K9" s="23" t="s">
+        <v>239</v>
+      </c>
+      <c r="L9" s="23" t="s">
+        <v>240</v>
+      </c>
+      <c r="M9" s="23" t="s">
+        <v>241</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="23" t="s">
+        <v>186</v>
+      </c>
+      <c r="B10" s="23">
+        <v>11.0</v>
+      </c>
+      <c r="C10" s="23">
+        <v>14.0</v>
+      </c>
+      <c r="D10" s="23" t="s">
+        <v>187</v>
+      </c>
+      <c r="E10" s="23">
+        <v>33.0</v>
+      </c>
+      <c r="F10" s="23">
+        <v>4.0</v>
+      </c>
+      <c r="G10" s="23">
+        <v>14.0</v>
+      </c>
+      <c r="H10" s="23" t="s">
+        <v>220</v>
+      </c>
+      <c r="I10" s="23" t="s">
+        <v>221</v>
+      </c>
+      <c r="J10" s="23" t="s">
+        <v>242</v>
+      </c>
+      <c r="K10" s="23" t="s">
+        <v>243</v>
+      </c>
+      <c r="L10" s="23" t="s">
+        <v>244</v>
+      </c>
+      <c r="M10" s="23" t="s">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="23" t="s">
+        <v>192</v>
+      </c>
+      <c r="B11" s="23">
+        <v>10.0</v>
+      </c>
+      <c r="C11" s="23">
+        <v>13.0</v>
+      </c>
+      <c r="D11" s="23" t="s">
+        <v>193</v>
+      </c>
+      <c r="E11" s="23">
+        <v>34.0</v>
+      </c>
+      <c r="F11" s="23">
+        <v>4.0</v>
+      </c>
+      <c r="G11" s="23">
+        <v>14.0</v>
+      </c>
+      <c r="H11" s="23" t="s">
+        <v>220</v>
+      </c>
+      <c r="I11" s="23" t="s">
+        <v>221</v>
+      </c>
+      <c r="J11" s="23" t="s">
+        <v>246</v>
+      </c>
+      <c r="K11" s="23" t="s">
+        <v>247</v>
+      </c>
+      <c r="L11" s="23" t="s">
+        <v>248</v>
+      </c>
+      <c r="M11" s="23" t="s">
+        <v>249</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="23" t="s">
+        <v>198</v>
+      </c>
+      <c r="B12" s="23">
+        <v>9.0</v>
+      </c>
+      <c r="C12" s="23">
+        <v>12.0</v>
+      </c>
+      <c r="D12" s="23" t="s">
+        <v>199</v>
+      </c>
+      <c r="E12" s="23">
         <v>35.0</v>
       </c>
-      <c r="C8" s="31">
-        <v>44.0</v>
-      </c>
-      <c r="D8" s="31" t="s">
-        <v>170</v>
-      </c>
-      <c r="E8" s="31">
-        <v>31.0</v>
-      </c>
-      <c r="F8" s="31">
+      <c r="F12" s="23">
+        <v>4.0</v>
+      </c>
+      <c r="G12" s="23">
+        <v>14.0</v>
+      </c>
+      <c r="H12" s="23" t="s">
+        <v>220</v>
+      </c>
+      <c r="I12" s="23" t="s">
+        <v>221</v>
+      </c>
+      <c r="J12" s="23" t="s">
+        <v>250</v>
+      </c>
+      <c r="K12" s="23" t="s">
+        <v>251</v>
+      </c>
+      <c r="L12" s="23" t="s">
+        <v>252</v>
+      </c>
+      <c r="M12" s="23" t="s">
+        <v>253</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="23" t="s">
+        <v>204</v>
+      </c>
+      <c r="B13" s="23">
         <v>6.0</v>
       </c>
-      <c r="G8" s="31">
-        <v>62.0</v>
-      </c>
-      <c r="H8" s="31" t="s">
-        <v>179</v>
-      </c>
-      <c r="I8" s="31" t="s">
-        <v>180</v>
-      </c>
-      <c r="J8" s="31" t="s">
-        <v>231</v>
-      </c>
-      <c r="K8" s="31" t="s">
-        <v>232</v>
-      </c>
-      <c r="L8" s="31" t="s">
-        <v>233</v>
-      </c>
-      <c r="M8" s="31" t="s">
-        <v>234</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="31" t="s">
-        <v>177</v>
-      </c>
-      <c r="B9" s="31">
-        <v>15.0</v>
-      </c>
-      <c r="C9" s="31">
-        <v>19.0</v>
-      </c>
-      <c r="D9" s="31" t="s">
-        <v>178</v>
-      </c>
-      <c r="E9" s="31">
-        <v>32.0</v>
-      </c>
-      <c r="F9" s="31">
-        <v>5.0</v>
-      </c>
-      <c r="G9" s="31">
-        <v>30.0</v>
-      </c>
-      <c r="H9" s="31" t="s">
+      <c r="C13" s="23">
+        <v>8.0</v>
+      </c>
+      <c r="D13" s="23" t="s">
         <v>205</v>
       </c>
-      <c r="I9" s="31" t="s">
-        <v>206</v>
-      </c>
-      <c r="J9" s="31" t="s">
-        <v>235</v>
-      </c>
-      <c r="K9" s="31" t="s">
-        <v>236</v>
-      </c>
-      <c r="L9" s="31" t="s">
-        <v>237</v>
-      </c>
-      <c r="M9" s="31" t="s">
-        <v>238</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="31" t="s">
-        <v>185</v>
-      </c>
-      <c r="B10" s="31">
-        <v>11.0</v>
-      </c>
-      <c r="C10" s="31">
+      <c r="E13" s="23">
+        <v>36.0</v>
+      </c>
+      <c r="F13" s="23">
+        <v>4.0</v>
+      </c>
+      <c r="G13" s="23">
         <v>14.0</v>
       </c>
-      <c r="D10" s="31" t="s">
-        <v>186</v>
-      </c>
-      <c r="E10" s="31">
-        <v>33.0</v>
-      </c>
-      <c r="F10" s="31">
-        <v>4.0</v>
-      </c>
-      <c r="G10" s="31">
-        <v>14.0</v>
-      </c>
-      <c r="H10" s="31" t="s">
+      <c r="H13" s="23" t="s">
+        <v>220</v>
+      </c>
+      <c r="I13" s="23" t="s">
+        <v>221</v>
+      </c>
+      <c r="J13" s="23" t="s">
+        <v>254</v>
+      </c>
+      <c r="K13" s="23" t="s">
+        <v>255</v>
+      </c>
+      <c r="L13" s="23" t="s">
+        <v>256</v>
+      </c>
+      <c r="M13" s="23" t="s">
+        <v>257</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="23" t="s">
+        <v>258</v>
+      </c>
+      <c r="B14" s="23">
+        <v>2.0</v>
+      </c>
+      <c r="C14" s="23">
+        <v>3.0</v>
+      </c>
+      <c r="D14" s="23" t="s">
+        <v>213</v>
+      </c>
+      <c r="E14" s="23">
+        <v>99.0</v>
+      </c>
+      <c r="F14" s="23">
+        <v>3.0</v>
+      </c>
+      <c r="G14" s="23">
+        <v>6.0</v>
+      </c>
+      <c r="H14" s="23" t="s">
+        <v>259</v>
+      </c>
+      <c r="I14" s="23" t="s">
+        <v>260</v>
+      </c>
+      <c r="J14" s="23" t="s">
+        <v>261</v>
+      </c>
+      <c r="K14" s="23" t="s">
+        <v>262</v>
+      </c>
+      <c r="L14" s="23" t="s">
+        <v>263</v>
+      </c>
+      <c r="M14" s="23" t="s">
+        <v>264</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="23" t="s">
+        <v>218</v>
+      </c>
+      <c r="B15" s="23">
+        <v>2.0</v>
+      </c>
+      <c r="C15" s="23">
+        <v>3.0</v>
+      </c>
+      <c r="D15" s="23" t="s">
         <v>219</v>
       </c>
-      <c r="I10" s="31" t="s">
-        <v>220</v>
-      </c>
-      <c r="J10" s="31" t="s">
-        <v>239</v>
-      </c>
-      <c r="K10" s="31" t="s">
-        <v>240</v>
-      </c>
-      <c r="L10" s="31" t="s">
-        <v>241</v>
-      </c>
-      <c r="M10" s="31" t="s">
-        <v>242</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="31" t="s">
-        <v>191</v>
-      </c>
-      <c r="B11" s="31">
-        <v>10.0</v>
-      </c>
-      <c r="C11" s="31">
-        <v>13.0</v>
-      </c>
-      <c r="D11" s="31" t="s">
-        <v>192</v>
-      </c>
-      <c r="E11" s="31">
-        <v>34.0</v>
-      </c>
-      <c r="F11" s="31">
-        <v>4.0</v>
-      </c>
-      <c r="G11" s="31">
-        <v>14.0</v>
-      </c>
-      <c r="H11" s="31" t="s">
-        <v>219</v>
-      </c>
-      <c r="I11" s="31" t="s">
-        <v>220</v>
-      </c>
-      <c r="J11" s="31" t="s">
-        <v>243</v>
-      </c>
-      <c r="K11" s="31" t="s">
-        <v>244</v>
-      </c>
-      <c r="L11" s="31" t="s">
-        <v>245</v>
-      </c>
-      <c r="M11" s="31" t="s">
-        <v>246</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="31" t="s">
-        <v>197</v>
-      </c>
-      <c r="B12" s="31">
-        <v>9.0</v>
-      </c>
-      <c r="C12" s="31">
-        <v>12.0</v>
-      </c>
-      <c r="D12" s="31" t="s">
-        <v>198</v>
-      </c>
-      <c r="E12" s="31">
-        <v>35.0</v>
-      </c>
-      <c r="F12" s="31">
-        <v>4.0</v>
-      </c>
-      <c r="G12" s="31">
-        <v>14.0</v>
-      </c>
-      <c r="H12" s="31" t="s">
-        <v>219</v>
-      </c>
-      <c r="I12" s="31" t="s">
-        <v>220</v>
-      </c>
-      <c r="J12" s="31" t="s">
-        <v>247</v>
-      </c>
-      <c r="K12" s="31" t="s">
-        <v>248</v>
-      </c>
-      <c r="L12" s="31" t="s">
-        <v>249</v>
-      </c>
-      <c r="M12" s="31" t="s">
-        <v>250</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="31" t="s">
-        <v>203</v>
-      </c>
-      <c r="B13" s="31">
+      <c r="E15" s="23">
+        <v>37.0</v>
+      </c>
+      <c r="F15" s="23">
+        <v>3.0</v>
+      </c>
+      <c r="G15" s="23">
         <v>6.0</v>
       </c>
-      <c r="C13" s="31">
-        <v>8.0</v>
-      </c>
-      <c r="D13" s="31" t="s">
-        <v>204</v>
-      </c>
-      <c r="E13" s="31">
-        <v>36.0</v>
-      </c>
-      <c r="F13" s="31">
-        <v>4.0</v>
-      </c>
-      <c r="G13" s="31">
-        <v>14.0</v>
-      </c>
-      <c r="H13" s="31" t="s">
-        <v>219</v>
-      </c>
-      <c r="I13" s="31" t="s">
-        <v>220</v>
-      </c>
-      <c r="J13" s="31" t="s">
-        <v>251</v>
-      </c>
-      <c r="K13" s="31" t="s">
-        <v>252</v>
-      </c>
-      <c r="L13" s="31" t="s">
-        <v>253</v>
-      </c>
-      <c r="M13" s="31" t="s">
-        <v>254</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="31" t="s">
-        <v>211</v>
-      </c>
-      <c r="B14" s="31">
-        <v>2.0</v>
-      </c>
-      <c r="C14" s="31">
-        <v>3.0</v>
-      </c>
-      <c r="D14" s="31" t="s">
-        <v>212</v>
-      </c>
-      <c r="E14" s="31">
-        <v>99.0</v>
-      </c>
-      <c r="F14" s="31">
-        <v>3.0</v>
-      </c>
-      <c r="G14" s="31">
-        <v>6.0</v>
-      </c>
-      <c r="H14" s="31" t="s">
-        <v>255</v>
-      </c>
-      <c r="I14" s="31" t="s">
-        <v>256</v>
-      </c>
-      <c r="J14" s="31" t="s">
-        <v>257</v>
-      </c>
-      <c r="K14" s="31" t="s">
-        <v>258</v>
-      </c>
-      <c r="L14" s="31" t="s">
+      <c r="H15" s="23" t="s">
         <v>259</v>
       </c>
-      <c r="M14" s="31" t="s">
+      <c r="I15" s="23" t="s">
         <v>260</v>
       </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="31" t="s">
-        <v>217</v>
-      </c>
-      <c r="B15" s="31">
-        <v>2.0</v>
-      </c>
-      <c r="C15" s="31">
-        <v>3.0</v>
-      </c>
-      <c r="D15" s="31" t="s">
-        <v>218</v>
-      </c>
-      <c r="E15" s="31">
-        <v>37.0</v>
-      </c>
-      <c r="F15" s="31">
-        <v>3.0</v>
-      </c>
-      <c r="G15" s="31">
-        <v>6.0</v>
-      </c>
-      <c r="H15" s="31" t="s">
-        <v>255</v>
-      </c>
-      <c r="I15" s="31" t="s">
-        <v>256</v>
-      </c>
-      <c r="J15" s="31" t="s">
-        <v>261</v>
-      </c>
-      <c r="K15" s="31" t="s">
-        <v>262</v>
-      </c>
-      <c r="L15" s="31" t="s">
-        <v>263</v>
-      </c>
-      <c r="M15" s="31" t="s">
-        <v>264</v>
+      <c r="J15" s="23" t="s">
+        <v>265</v>
+      </c>
+      <c r="K15" s="23" t="s">
+        <v>266</v>
+      </c>
+      <c r="L15" s="23" t="s">
+        <v>267</v>
+      </c>
+      <c r="M15" s="23" t="s">
+        <v>268</v>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="25" t="s">
-        <v>225</v>
-      </c>
-      <c r="B16" s="32">
+      <c r="A16" s="24" t="s">
+        <v>269</v>
+      </c>
+      <c r="B16" s="29">
         <f>SUM(B7:B15)</f>
         <v>160</v>
       </c>
-      <c r="C16" s="32">
+      <c r="C16" s="29">
         <v>204.0</v>
       </c>
       <c r="D16" s="28"/>
       <c r="E16" s="28"/>
       <c r="F16" s="28"/>
-      <c r="G16" s="32">
+      <c r="G16" s="29">
         <v>286.0</v>
       </c>
       <c r="H16" s="28"/>
@@ -3626,11 +3655,11 @@
       <c r="M17" s="28"/>
     </row>
     <row r="18">
-      <c r="A18" s="25" t="s">
-        <v>265</v>
-      </c>
-      <c r="B18" s="29" t="s">
-        <v>266</v>
+      <c r="A18" s="24" t="s">
+        <v>228</v>
+      </c>
+      <c r="B18" s="25" t="s">
+        <v>270</v>
       </c>
       <c r="C18" s="28"/>
       <c r="D18" s="28"/>
@@ -3660,9 +3689,6 @@
       <c r="M19" s="28"/>
     </row>
   </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="B1:D1"/>
-  </mergeCells>
   <drawing r:id="rId1"/>
 </worksheet>
 </file>
@@ -3688,14 +3714,14 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="25" t="s">
+      <c r="A1" s="24" t="s">
         <v>150</v>
       </c>
-      <c r="B1" s="26" t="s">
-        <v>267</v>
-      </c>
-      <c r="C1" s="27"/>
-      <c r="D1" s="18"/>
+      <c r="B1" s="25" t="s">
+        <v>271</v>
+      </c>
+      <c r="C1" s="26"/>
+      <c r="D1" s="27"/>
       <c r="E1" s="28"/>
       <c r="F1" s="28"/>
       <c r="G1" s="28"/>
@@ -3845,13 +3871,13 @@
       <c r="EU1" s="28"/>
     </row>
     <row r="2">
-      <c r="A2" s="25" t="s">
+      <c r="A2" s="24" t="s">
         <v>77</v>
       </c>
-      <c r="B2" s="29" t="s">
+      <c r="B2" s="25" t="s">
         <v>110</v>
       </c>
-      <c r="C2" s="33"/>
+      <c r="C2" s="30"/>
       <c r="D2" s="28"/>
       <c r="E2" s="28"/>
       <c r="F2" s="28"/>
@@ -4002,13 +4028,13 @@
       <c r="EU2" s="28"/>
     </row>
     <row r="3">
-      <c r="A3" s="25" t="s">
+      <c r="A3" s="24" t="s">
         <v>79</v>
       </c>
-      <c r="B3" s="29" t="s">
-        <v>268</v>
-      </c>
-      <c r="C3" s="33"/>
+      <c r="B3" s="25" t="s">
+        <v>272</v>
+      </c>
+      <c r="C3" s="30"/>
       <c r="D3" s="28"/>
       <c r="E3" s="28"/>
       <c r="F3" s="28"/>
@@ -4465,44 +4491,44 @@
       <c r="EU5" s="28"/>
     </row>
     <row r="6">
-      <c r="A6" s="30" t="s">
+      <c r="A6" s="22" t="s">
         <v>155</v>
       </c>
-      <c r="B6" s="30" t="s">
+      <c r="B6" s="22" t="s">
         <v>156</v>
       </c>
-      <c r="C6" s="30" t="s">
+      <c r="C6" s="22" t="s">
         <v>157</v>
       </c>
-      <c r="D6" s="30" t="s">
+      <c r="D6" s="22" t="s">
         <v>158</v>
       </c>
-      <c r="E6" s="30" t="s">
+      <c r="E6" s="22" t="s">
         <v>159</v>
       </c>
-      <c r="F6" s="30" t="s">
+      <c r="F6" s="22" t="s">
         <v>160</v>
       </c>
-      <c r="G6" s="30" t="s">
+      <c r="G6" s="22" t="s">
         <v>161</v>
       </c>
-      <c r="H6" s="30" t="s">
+      <c r="H6" s="22" t="s">
         <v>14</v>
       </c>
-      <c r="I6" s="30" t="s">
+      <c r="I6" s="22" t="s">
         <v>162</v>
       </c>
-      <c r="J6" s="30" t="s">
+      <c r="J6" s="22" t="s">
         <v>127</v>
       </c>
-      <c r="K6" s="30" t="s">
+      <c r="K6" s="22" t="s">
         <v>15</v>
       </c>
-      <c r="L6" s="30" t="s">
+      <c r="L6" s="22" t="s">
         <v>16</v>
       </c>
-      <c r="M6" s="30" t="s">
-        <v>228</v>
+      <c r="M6" s="22" t="s">
+        <v>163</v>
       </c>
       <c r="N6" s="28"/>
       <c r="O6" s="28"/>
@@ -4644,44 +4670,44 @@
       <c r="EU6" s="28"/>
     </row>
     <row r="7" ht="24.75" customHeight="1">
-      <c r="A7" s="31" t="s">
-        <v>163</v>
-      </c>
-      <c r="B7" s="31">
+      <c r="A7" s="23" t="s">
+        <v>164</v>
+      </c>
+      <c r="B7" s="23">
         <v>78.0</v>
       </c>
-      <c r="C7" s="31">
+      <c r="C7" s="23">
         <v>98.0</v>
       </c>
-      <c r="D7" s="31" t="s">
-        <v>164</v>
-      </c>
-      <c r="E7" s="31">
+      <c r="D7" s="23" t="s">
+        <v>165</v>
+      </c>
+      <c r="E7" s="23">
         <v>20.0</v>
       </c>
-      <c r="F7" s="31">
+      <c r="F7" s="23">
         <v>7.0</v>
       </c>
-      <c r="G7" s="31">
+      <c r="G7" s="23">
         <v>126.0</v>
       </c>
-      <c r="H7" s="31" t="s">
-        <v>171</v>
-      </c>
-      <c r="I7" s="31" t="s">
+      <c r="H7" s="23" t="s">
         <v>172</v>
       </c>
-      <c r="J7" s="31" t="s">
+      <c r="I7" s="23" t="s">
+        <v>173</v>
+      </c>
+      <c r="J7" s="23" t="s">
         <v>106</v>
       </c>
-      <c r="K7" s="31" t="s">
+      <c r="K7" s="23" t="s">
         <v>107</v>
       </c>
-      <c r="L7" s="31" t="s">
-        <v>269</v>
-      </c>
-      <c r="M7" s="31" t="s">
-        <v>270</v>
+      <c r="L7" s="23" t="s">
+        <v>273</v>
+      </c>
+      <c r="M7" s="23" t="s">
+        <v>274</v>
       </c>
       <c r="N7" s="28"/>
       <c r="O7" s="28"/>
@@ -4823,44 +4849,44 @@
       <c r="EU7" s="28"/>
     </row>
     <row r="8" ht="22.5" customHeight="1">
-      <c r="A8" s="31" t="s">
-        <v>169</v>
-      </c>
-      <c r="B8" s="31">
+      <c r="A8" s="23" t="s">
+        <v>170</v>
+      </c>
+      <c r="B8" s="23">
         <v>40.0</v>
       </c>
-      <c r="C8" s="31">
+      <c r="C8" s="23">
         <v>50.0</v>
       </c>
-      <c r="D8" s="31" t="s">
-        <v>170</v>
-      </c>
-      <c r="E8" s="31">
+      <c r="D8" s="23" t="s">
+        <v>171</v>
+      </c>
+      <c r="E8" s="23">
         <v>21.0</v>
       </c>
-      <c r="F8" s="31">
+      <c r="F8" s="23">
         <v>6.0</v>
       </c>
-      <c r="G8" s="31">
+      <c r="G8" s="23">
         <v>62.0</v>
       </c>
-      <c r="H8" s="31" t="s">
-        <v>179</v>
-      </c>
-      <c r="I8" s="31" t="s">
+      <c r="H8" s="23" t="s">
         <v>180</v>
       </c>
-      <c r="J8" s="31" t="s">
-        <v>271</v>
-      </c>
-      <c r="K8" s="31" t="s">
-        <v>272</v>
-      </c>
-      <c r="L8" s="31" t="s">
-        <v>273</v>
-      </c>
-      <c r="M8" s="31" t="s">
-        <v>274</v>
+      <c r="I8" s="23" t="s">
+        <v>181</v>
+      </c>
+      <c r="J8" s="23" t="s">
+        <v>275</v>
+      </c>
+      <c r="K8" s="23" t="s">
+        <v>276</v>
+      </c>
+      <c r="L8" s="23" t="s">
+        <v>277</v>
+      </c>
+      <c r="M8" s="23" t="s">
+        <v>278</v>
       </c>
       <c r="N8" s="28"/>
       <c r="O8" s="28"/>
@@ -5002,44 +5028,44 @@
       <c r="EU8" s="28"/>
     </row>
     <row r="9">
-      <c r="A9" s="31" t="s">
-        <v>177</v>
-      </c>
-      <c r="B9" s="31">
+      <c r="A9" s="23" t="s">
+        <v>178</v>
+      </c>
+      <c r="B9" s="23">
         <v>16.0</v>
       </c>
-      <c r="C9" s="31">
+      <c r="C9" s="23">
         <v>20.0</v>
       </c>
-      <c r="D9" s="31" t="s">
-        <v>178</v>
-      </c>
-      <c r="E9" s="31">
+      <c r="D9" s="23" t="s">
+        <v>179</v>
+      </c>
+      <c r="E9" s="23">
         <v>22.0</v>
       </c>
-      <c r="F9" s="31">
+      <c r="F9" s="23">
         <v>5.0</v>
       </c>
-      <c r="G9" s="31">
+      <c r="G9" s="23">
         <v>30.0</v>
       </c>
-      <c r="H9" s="31" t="s">
-        <v>205</v>
-      </c>
-      <c r="I9" s="31" t="s">
+      <c r="H9" s="23" t="s">
         <v>206</v>
       </c>
-      <c r="J9" s="31" t="s">
-        <v>275</v>
-      </c>
-      <c r="K9" s="31" t="s">
-        <v>276</v>
-      </c>
-      <c r="L9" s="31" t="s">
-        <v>277</v>
-      </c>
-      <c r="M9" s="31" t="s">
-        <v>278</v>
+      <c r="I9" s="23" t="s">
+        <v>207</v>
+      </c>
+      <c r="J9" s="23" t="s">
+        <v>279</v>
+      </c>
+      <c r="K9" s="23" t="s">
+        <v>280</v>
+      </c>
+      <c r="L9" s="23" t="s">
+        <v>281</v>
+      </c>
+      <c r="M9" s="23" t="s">
+        <v>282</v>
       </c>
       <c r="N9" s="28"/>
       <c r="O9" s="28"/>
@@ -5181,44 +5207,44 @@
       <c r="EU9" s="28"/>
     </row>
     <row r="10">
-      <c r="A10" s="31" t="s">
-        <v>185</v>
-      </c>
-      <c r="B10" s="31">
+      <c r="A10" s="23" t="s">
+        <v>186</v>
+      </c>
+      <c r="B10" s="23">
         <v>12.0</v>
       </c>
-      <c r="C10" s="31">
+      <c r="C10" s="23">
         <v>15.0</v>
       </c>
-      <c r="D10" s="31" t="s">
-        <v>186</v>
-      </c>
-      <c r="E10" s="31">
+      <c r="D10" s="23" t="s">
+        <v>187</v>
+      </c>
+      <c r="E10" s="23">
         <v>23.0</v>
       </c>
-      <c r="F10" s="31">
+      <c r="F10" s="23">
         <v>5.0</v>
       </c>
-      <c r="G10" s="31">
+      <c r="G10" s="23">
         <v>30.0</v>
       </c>
-      <c r="H10" s="31" t="s">
-        <v>205</v>
-      </c>
-      <c r="I10" s="31" t="s">
+      <c r="H10" s="23" t="s">
         <v>206</v>
       </c>
-      <c r="J10" s="31" t="s">
-        <v>279</v>
-      </c>
-      <c r="K10" s="31" t="s">
-        <v>280</v>
-      </c>
-      <c r="L10" s="31" t="s">
-        <v>281</v>
-      </c>
-      <c r="M10" s="31" t="s">
-        <v>282</v>
+      <c r="I10" s="23" t="s">
+        <v>207</v>
+      </c>
+      <c r="J10" s="23" t="s">
+        <v>283</v>
+      </c>
+      <c r="K10" s="23" t="s">
+        <v>284</v>
+      </c>
+      <c r="L10" s="23" t="s">
+        <v>285</v>
+      </c>
+      <c r="M10" s="23" t="s">
+        <v>286</v>
       </c>
       <c r="N10" s="28"/>
       <c r="O10" s="28"/>
@@ -5360,44 +5386,44 @@
       <c r="EU10" s="28"/>
     </row>
     <row r="11">
-      <c r="A11" s="31" t="s">
-        <v>191</v>
-      </c>
-      <c r="B11" s="31">
+      <c r="A11" s="23" t="s">
+        <v>192</v>
+      </c>
+      <c r="B11" s="23">
         <v>11.0</v>
       </c>
-      <c r="C11" s="31">
+      <c r="C11" s="23">
         <v>14.0</v>
       </c>
-      <c r="D11" s="31" t="s">
-        <v>192</v>
-      </c>
-      <c r="E11" s="31">
+      <c r="D11" s="23" t="s">
+        <v>193</v>
+      </c>
+      <c r="E11" s="23">
         <v>24.0</v>
       </c>
-      <c r="F11" s="31">
+      <c r="F11" s="23">
         <v>4.0</v>
       </c>
-      <c r="G11" s="31">
+      <c r="G11" s="23">
         <v>14.0</v>
       </c>
-      <c r="H11" s="31" t="s">
-        <v>219</v>
-      </c>
-      <c r="I11" s="31" t="s">
+      <c r="H11" s="23" t="s">
         <v>220</v>
       </c>
-      <c r="J11" s="31" t="s">
-        <v>283</v>
-      </c>
-      <c r="K11" s="31" t="s">
-        <v>284</v>
-      </c>
-      <c r="L11" s="31" t="s">
-        <v>285</v>
-      </c>
-      <c r="M11" s="31" t="s">
-        <v>286</v>
+      <c r="I11" s="23" t="s">
+        <v>221</v>
+      </c>
+      <c r="J11" s="23" t="s">
+        <v>287</v>
+      </c>
+      <c r="K11" s="23" t="s">
+        <v>288</v>
+      </c>
+      <c r="L11" s="23" t="s">
+        <v>289</v>
+      </c>
+      <c r="M11" s="23" t="s">
+        <v>290</v>
       </c>
       <c r="N11" s="28"/>
       <c r="O11" s="28"/>
@@ -5539,44 +5565,44 @@
       <c r="EU11" s="28"/>
     </row>
     <row r="12">
-      <c r="A12" s="31" t="s">
-        <v>197</v>
-      </c>
-      <c r="B12" s="31">
+      <c r="A12" s="23" t="s">
+        <v>198</v>
+      </c>
+      <c r="B12" s="23">
         <v>10.0</v>
       </c>
-      <c r="C12" s="31">
+      <c r="C12" s="23">
         <v>13.0</v>
       </c>
-      <c r="D12" s="31" t="s">
-        <v>198</v>
-      </c>
-      <c r="E12" s="31">
+      <c r="D12" s="23" t="s">
+        <v>199</v>
+      </c>
+      <c r="E12" s="23">
         <v>25.0</v>
       </c>
-      <c r="F12" s="31">
+      <c r="F12" s="23">
         <v>4.0</v>
       </c>
-      <c r="G12" s="31">
+      <c r="G12" s="23">
         <v>14.0</v>
       </c>
-      <c r="H12" s="31" t="s">
-        <v>219</v>
-      </c>
-      <c r="I12" s="31" t="s">
+      <c r="H12" s="23" t="s">
         <v>220</v>
       </c>
-      <c r="J12" s="31" t="s">
-        <v>287</v>
-      </c>
-      <c r="K12" s="31" t="s">
-        <v>288</v>
-      </c>
-      <c r="L12" s="31" t="s">
-        <v>289</v>
-      </c>
-      <c r="M12" s="31" t="s">
-        <v>290</v>
+      <c r="I12" s="23" t="s">
+        <v>221</v>
+      </c>
+      <c r="J12" s="23" t="s">
+        <v>291</v>
+      </c>
+      <c r="K12" s="23" t="s">
+        <v>292</v>
+      </c>
+      <c r="L12" s="23" t="s">
+        <v>293</v>
+      </c>
+      <c r="M12" s="23" t="s">
+        <v>294</v>
       </c>
       <c r="N12" s="28"/>
       <c r="O12" s="28"/>
@@ -5718,44 +5744,44 @@
       <c r="EU12" s="28"/>
     </row>
     <row r="13">
-      <c r="A13" s="31" t="s">
-        <v>211</v>
-      </c>
-      <c r="B13" s="31">
+      <c r="A13" s="23" t="s">
+        <v>258</v>
+      </c>
+      <c r="B13" s="23">
         <v>10.0</v>
       </c>
-      <c r="C13" s="31">
+      <c r="C13" s="23">
         <v>13.0</v>
       </c>
-      <c r="D13" s="31" t="s">
-        <v>212</v>
-      </c>
-      <c r="E13" s="31">
+      <c r="D13" s="23" t="s">
+        <v>213</v>
+      </c>
+      <c r="E13" s="23">
         <v>99.0</v>
       </c>
-      <c r="F13" s="31">
+      <c r="F13" s="23">
         <v>4.0</v>
       </c>
-      <c r="G13" s="31">
+      <c r="G13" s="23">
         <v>14.0</v>
       </c>
-      <c r="H13" s="31" t="s">
-        <v>219</v>
-      </c>
-      <c r="I13" s="31" t="s">
+      <c r="H13" s="23" t="s">
         <v>220</v>
       </c>
-      <c r="J13" s="31" t="s">
-        <v>291</v>
-      </c>
-      <c r="K13" s="31" t="s">
-        <v>292</v>
-      </c>
-      <c r="L13" s="31" t="s">
-        <v>293</v>
-      </c>
-      <c r="M13" s="31" t="s">
-        <v>294</v>
+      <c r="I13" s="23" t="s">
+        <v>221</v>
+      </c>
+      <c r="J13" s="23" t="s">
+        <v>295</v>
+      </c>
+      <c r="K13" s="23" t="s">
+        <v>296</v>
+      </c>
+      <c r="L13" s="23" t="s">
+        <v>297</v>
+      </c>
+      <c r="M13" s="23" t="s">
+        <v>298</v>
       </c>
       <c r="N13" s="28"/>
       <c r="O13" s="28"/>
@@ -5897,44 +5923,44 @@
       <c r="EU13" s="28"/>
     </row>
     <row r="14">
-      <c r="A14" s="31" t="s">
-        <v>203</v>
-      </c>
-      <c r="B14" s="31">
+      <c r="A14" s="23" t="s">
+        <v>204</v>
+      </c>
+      <c r="B14" s="23">
         <v>8.0</v>
       </c>
-      <c r="C14" s="31">
+      <c r="C14" s="23">
         <v>10.0</v>
       </c>
-      <c r="D14" s="31" t="s">
-        <v>204</v>
-      </c>
-      <c r="E14" s="31">
+      <c r="D14" s="23" t="s">
+        <v>205</v>
+      </c>
+      <c r="E14" s="23">
         <v>26.0</v>
       </c>
-      <c r="F14" s="31">
+      <c r="F14" s="23">
         <v>4.0</v>
       </c>
-      <c r="G14" s="31">
+      <c r="G14" s="23">
         <v>14.0</v>
       </c>
-      <c r="H14" s="31" t="s">
-        <v>219</v>
-      </c>
-      <c r="I14" s="31" t="s">
+      <c r="H14" s="23" t="s">
         <v>220</v>
       </c>
-      <c r="J14" s="31" t="s">
-        <v>295</v>
-      </c>
-      <c r="K14" s="31" t="s">
-        <v>296</v>
-      </c>
-      <c r="L14" s="31" t="s">
-        <v>297</v>
-      </c>
-      <c r="M14" s="31" t="s">
-        <v>298</v>
+      <c r="I14" s="23" t="s">
+        <v>221</v>
+      </c>
+      <c r="J14" s="23" t="s">
+        <v>299</v>
+      </c>
+      <c r="K14" s="23" t="s">
+        <v>300</v>
+      </c>
+      <c r="L14" s="23" t="s">
+        <v>301</v>
+      </c>
+      <c r="M14" s="23" t="s">
+        <v>302</v>
       </c>
       <c r="N14" s="28"/>
       <c r="O14" s="28"/>
@@ -6076,44 +6102,44 @@
       <c r="EU14" s="28"/>
     </row>
     <row r="15">
-      <c r="A15" s="31" t="s">
-        <v>217</v>
-      </c>
-      <c r="B15" s="31">
+      <c r="A15" s="23" t="s">
+        <v>218</v>
+      </c>
+      <c r="B15" s="23">
         <v>5.0</v>
       </c>
-      <c r="C15" s="31">
+      <c r="C15" s="23">
         <v>7.0</v>
       </c>
-      <c r="D15" s="31" t="s">
-        <v>218</v>
-      </c>
-      <c r="E15" s="31">
+      <c r="D15" s="23" t="s">
+        <v>219</v>
+      </c>
+      <c r="E15" s="23">
         <v>27.0</v>
       </c>
-      <c r="F15" s="31">
+      <c r="F15" s="23">
         <v>4.0</v>
       </c>
-      <c r="G15" s="31">
+      <c r="G15" s="23">
         <v>14.0</v>
       </c>
-      <c r="H15" s="31" t="s">
-        <v>219</v>
-      </c>
-      <c r="I15" s="31" t="s">
+      <c r="H15" s="23" t="s">
         <v>220</v>
       </c>
-      <c r="J15" s="31" t="s">
-        <v>299</v>
-      </c>
-      <c r="K15" s="31" t="s">
-        <v>300</v>
-      </c>
-      <c r="L15" s="31" t="s">
-        <v>301</v>
-      </c>
-      <c r="M15" s="31" t="s">
-        <v>302</v>
+      <c r="I15" s="23" t="s">
+        <v>221</v>
+      </c>
+      <c r="J15" s="23" t="s">
+        <v>303</v>
+      </c>
+      <c r="K15" s="23" t="s">
+        <v>304</v>
+      </c>
+      <c r="L15" s="23" t="s">
+        <v>305</v>
+      </c>
+      <c r="M15" s="23" t="s">
+        <v>306</v>
       </c>
       <c r="N15" s="28"/>
       <c r="O15" s="28"/>
@@ -6255,25 +6281,25 @@
       <c r="EU15" s="28"/>
     </row>
     <row r="16">
-      <c r="A16" s="25" t="s">
-        <v>225</v>
-      </c>
-      <c r="B16" s="32">
+      <c r="A16" s="24" t="s">
+        <v>269</v>
+      </c>
+      <c r="B16" s="29">
         <v>190.0</v>
       </c>
-      <c r="C16" s="32">
+      <c r="C16" s="29">
         <v>240.0</v>
       </c>
-      <c r="D16" s="33"/>
-      <c r="E16" s="33"/>
-      <c r="F16" s="33"/>
-      <c r="G16" s="32">
+      <c r="D16" s="30"/>
+      <c r="E16" s="30"/>
+      <c r="F16" s="30"/>
+      <c r="G16" s="29">
         <v>318.0</v>
       </c>
-      <c r="H16" s="33"/>
-      <c r="I16" s="33"/>
-      <c r="J16" s="33"/>
-      <c r="K16" s="33"/>
+      <c r="H16" s="30"/>
+      <c r="I16" s="30"/>
+      <c r="J16" s="30"/>
+      <c r="K16" s="30"/>
       <c r="L16" s="28"/>
       <c r="M16" s="28"/>
       <c r="N16" s="28"/>
@@ -6416,17 +6442,17 @@
       <c r="EU16" s="28"/>
     </row>
     <row r="17">
-      <c r="A17" s="33"/>
-      <c r="B17" s="33"/>
-      <c r="C17" s="33"/>
-      <c r="D17" s="33"/>
-      <c r="E17" s="33"/>
-      <c r="F17" s="33"/>
-      <c r="G17" s="33"/>
-      <c r="H17" s="33"/>
-      <c r="I17" s="33"/>
-      <c r="J17" s="33"/>
-      <c r="K17" s="33"/>
+      <c r="A17" s="30"/>
+      <c r="B17" s="30"/>
+      <c r="C17" s="30"/>
+      <c r="D17" s="30"/>
+      <c r="E17" s="30"/>
+      <c r="F17" s="30"/>
+      <c r="G17" s="30"/>
+      <c r="H17" s="30"/>
+      <c r="I17" s="30"/>
+      <c r="J17" s="30"/>
+      <c r="K17" s="30"/>
       <c r="L17" s="28"/>
       <c r="M17" s="28"/>
       <c r="N17" s="28"/>
@@ -6569,13 +6595,13 @@
       <c r="EU17" s="28"/>
     </row>
     <row r="18">
-      <c r="A18" s="25" t="s">
-        <v>265</v>
-      </c>
-      <c r="B18" s="29" t="s">
-        <v>303</v>
-      </c>
-      <c r="C18" s="33"/>
+      <c r="A18" s="24" t="s">
+        <v>228</v>
+      </c>
+      <c r="B18" s="25" t="s">
+        <v>307</v>
+      </c>
+      <c r="C18" s="30"/>
       <c r="D18" s="28"/>
       <c r="E18" s="28"/>
       <c r="F18" s="28"/>
@@ -6726,12 +6752,9 @@
       <c r="EU18" s="28"/>
     </row>
     <row r="19">
-      <c r="J19" s="34"/>
+      <c r="J19" s="31"/>
     </row>
   </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="B1:D1"/>
-  </mergeCells>
   <drawing r:id="rId1"/>
 </worksheet>
 </file>
@@ -6749,14 +6772,14 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="25" t="s">
+      <c r="A1" s="24" t="s">
         <v>150</v>
       </c>
-      <c r="B1" s="26" t="s">
-        <v>304</v>
-      </c>
-      <c r="C1" s="27"/>
-      <c r="D1" s="18"/>
+      <c r="B1" s="25" t="s">
+        <v>308</v>
+      </c>
+      <c r="C1" s="26"/>
+      <c r="D1" s="27"/>
       <c r="E1" s="28"/>
       <c r="F1" s="28"/>
       <c r="G1" s="28"/>
@@ -6768,13 +6791,13 @@
       <c r="M1" s="28"/>
     </row>
     <row r="2">
-      <c r="A2" s="25" t="s">
+      <c r="A2" s="24" t="s">
         <v>77</v>
       </c>
-      <c r="B2" s="29" t="s">
+      <c r="B2" s="25" t="s">
         <v>116</v>
       </c>
-      <c r="C2" s="33"/>
+      <c r="C2" s="30"/>
       <c r="D2" s="28"/>
       <c r="E2" s="28"/>
       <c r="F2" s="28"/>
@@ -6787,13 +6810,13 @@
       <c r="M2" s="28"/>
     </row>
     <row r="3">
-      <c r="A3" s="25" t="s">
+      <c r="A3" s="24" t="s">
         <v>79</v>
       </c>
-      <c r="B3" s="29" t="s">
-        <v>305</v>
-      </c>
-      <c r="C3" s="33"/>
+      <c r="B3" s="25" t="s">
+        <v>309</v>
+      </c>
+      <c r="C3" s="30"/>
       <c r="D3" s="28"/>
       <c r="E3" s="28"/>
       <c r="F3" s="28"/>
@@ -6835,430 +6858,439 @@
       <c r="L5" s="28"/>
       <c r="M5" s="28"/>
     </row>
-    <row r="6">
-      <c r="A6" s="30" t="s">
+    <row r="6" ht="51.75" customHeight="1">
+      <c r="A6" s="32" t="s">
         <v>155</v>
       </c>
-      <c r="B6" s="30" t="s">
+      <c r="B6" s="32" t="s">
         <v>156</v>
       </c>
-      <c r="C6" s="30" t="s">
+      <c r="C6" s="32" t="s">
         <v>157</v>
       </c>
-      <c r="D6" s="30" t="s">
+      <c r="D6" s="32" t="s">
         <v>158</v>
       </c>
-      <c r="E6" s="30" t="s">
+      <c r="E6" s="32" t="s">
         <v>159</v>
       </c>
-      <c r="F6" s="30" t="s">
+      <c r="F6" s="32" t="s">
         <v>160</v>
       </c>
-      <c r="G6" s="30" t="s">
+      <c r="G6" s="32" t="s">
         <v>161</v>
       </c>
-      <c r="H6" s="30" t="s">
+      <c r="H6" s="32" t="s">
         <v>14</v>
       </c>
-      <c r="I6" s="30" t="s">
+      <c r="I6" s="32" t="s">
         <v>162</v>
       </c>
-      <c r="J6" s="30" t="s">
+      <c r="J6" s="32" t="s">
         <v>127</v>
       </c>
-      <c r="K6" s="30" t="s">
+      <c r="K6" s="32" t="s">
         <v>15</v>
       </c>
-      <c r="L6" s="30" t="s">
+      <c r="L6" s="32" t="s">
         <v>16</v>
       </c>
-      <c r="M6" s="30" t="s">
-        <v>228</v>
+      <c r="M6" s="32" t="s">
+        <v>163</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="31" t="s">
-        <v>163</v>
-      </c>
-      <c r="B7" s="31">
-        <v>35.0</v>
-      </c>
-      <c r="C7" s="31">
+      <c r="A7" s="23" t="s">
+        <v>164</v>
+      </c>
+      <c r="B7" s="23">
+        <v>20.0</v>
+      </c>
+      <c r="C7" s="33">
+        <f t="shared" ref="C7:C15" si="1">B7*1.25</f>
+        <v>25</v>
+      </c>
+      <c r="D7" s="23" t="s">
+        <v>165</v>
+      </c>
+      <c r="E7" s="23">
+        <v>40.0</v>
+      </c>
+      <c r="F7" s="23">
+        <v>5.0</v>
+      </c>
+      <c r="G7" s="23">
+        <v>30.0</v>
+      </c>
+      <c r="H7" s="23" t="s">
+        <v>206</v>
+      </c>
+      <c r="I7" s="23" t="s">
+        <v>207</v>
+      </c>
+      <c r="J7" s="23" t="s">
+        <v>112</v>
+      </c>
+      <c r="K7" s="23" t="s">
+        <v>113</v>
+      </c>
+      <c r="L7" s="23" t="s">
+        <v>310</v>
+      </c>
+      <c r="M7" s="23" t="s">
+        <v>311</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="23" t="s">
+        <v>170</v>
+      </c>
+      <c r="B8" s="23">
+        <v>13.0</v>
+      </c>
+      <c r="C8" s="33">
+        <f t="shared" si="1"/>
+        <v>16.25</v>
+      </c>
+      <c r="D8" s="23" t="s">
+        <v>171</v>
+      </c>
+      <c r="E8" s="23">
+        <v>41.0</v>
+      </c>
+      <c r="F8" s="23">
+        <v>5.0</v>
+      </c>
+      <c r="G8" s="23">
+        <v>30.0</v>
+      </c>
+      <c r="H8" s="23" t="s">
+        <v>206</v>
+      </c>
+      <c r="I8" s="23" t="s">
+        <v>207</v>
+      </c>
+      <c r="J8" s="23" t="s">
+        <v>312</v>
+      </c>
+      <c r="K8" s="23" t="s">
+        <v>313</v>
+      </c>
+      <c r="L8" s="23" t="s">
+        <v>314</v>
+      </c>
+      <c r="M8" s="23" t="s">
+        <v>315</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="23" t="s">
+        <v>178</v>
+      </c>
+      <c r="B9" s="23">
+        <v>12.0</v>
+      </c>
+      <c r="C9" s="33">
+        <f t="shared" si="1"/>
+        <v>15</v>
+      </c>
+      <c r="D9" s="23" t="s">
+        <v>179</v>
+      </c>
+      <c r="E9" s="23">
+        <v>42.0</v>
+      </c>
+      <c r="F9" s="23">
+        <v>5.0</v>
+      </c>
+      <c r="G9" s="23">
+        <v>30.0</v>
+      </c>
+      <c r="H9" s="23" t="s">
+        <v>206</v>
+      </c>
+      <c r="I9" s="23" t="s">
+        <v>207</v>
+      </c>
+      <c r="J9" s="23" t="s">
+        <v>316</v>
+      </c>
+      <c r="K9" s="23" t="s">
+        <v>317</v>
+      </c>
+      <c r="L9" s="23" t="s">
+        <v>318</v>
+      </c>
+      <c r="M9" s="23" t="s">
+        <v>319</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="23" t="s">
+        <v>186</v>
+      </c>
+      <c r="B10" s="23">
+        <v>11.0</v>
+      </c>
+      <c r="C10" s="33">
+        <f t="shared" si="1"/>
+        <v>13.75</v>
+      </c>
+      <c r="D10" s="23" t="s">
+        <v>187</v>
+      </c>
+      <c r="E10" s="23">
+        <v>43.0</v>
+      </c>
+      <c r="F10" s="23">
+        <v>4.0</v>
+      </c>
+      <c r="G10" s="23">
+        <v>14.0</v>
+      </c>
+      <c r="H10" s="23" t="s">
+        <v>220</v>
+      </c>
+      <c r="I10" s="23" t="s">
+        <v>221</v>
+      </c>
+      <c r="J10" s="23" t="s">
+        <v>320</v>
+      </c>
+      <c r="K10" s="23" t="s">
+        <v>321</v>
+      </c>
+      <c r="L10" s="23" t="s">
+        <v>322</v>
+      </c>
+      <c r="M10" s="23" t="s">
+        <v>323</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="23" t="s">
+        <v>192</v>
+      </c>
+      <c r="B11" s="23">
+        <v>10.0</v>
+      </c>
+      <c r="C11" s="33">
+        <f t="shared" si="1"/>
+        <v>12.5</v>
+      </c>
+      <c r="D11" s="23" t="s">
+        <v>193</v>
+      </c>
+      <c r="E11" s="23">
         <v>44.0</v>
       </c>
-      <c r="D7" s="31" t="s">
-        <v>164</v>
-      </c>
-      <c r="E7" s="31">
-        <v>40.0</v>
-      </c>
-      <c r="F7" s="31">
+      <c r="F11" s="23">
+        <v>4.0</v>
+      </c>
+      <c r="G11" s="23">
+        <v>14.0</v>
+      </c>
+      <c r="H11" s="23" t="s">
+        <v>220</v>
+      </c>
+      <c r="I11" s="23" t="s">
+        <v>221</v>
+      </c>
+      <c r="J11" s="23" t="s">
+        <v>324</v>
+      </c>
+      <c r="K11" s="23" t="s">
+        <v>325</v>
+      </c>
+      <c r="L11" s="23" t="s">
+        <v>326</v>
+      </c>
+      <c r="M11" s="23" t="s">
+        <v>327</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="23" t="s">
+        <v>198</v>
+      </c>
+      <c r="B12" s="23">
+        <v>9.0</v>
+      </c>
+      <c r="C12" s="33">
+        <f t="shared" si="1"/>
+        <v>11.25</v>
+      </c>
+      <c r="D12" s="23" t="s">
+        <v>199</v>
+      </c>
+      <c r="E12" s="23">
+        <v>45.0</v>
+      </c>
+      <c r="F12" s="23">
+        <v>4.0</v>
+      </c>
+      <c r="G12" s="23">
+        <v>14.0</v>
+      </c>
+      <c r="H12" s="23" t="s">
+        <v>220</v>
+      </c>
+      <c r="I12" s="23" t="s">
+        <v>221</v>
+      </c>
+      <c r="J12" s="23" t="s">
+        <v>328</v>
+      </c>
+      <c r="K12" s="23" t="s">
+        <v>329</v>
+      </c>
+      <c r="L12" s="23" t="s">
+        <v>330</v>
+      </c>
+      <c r="M12" s="23" t="s">
+        <v>331</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="23" t="s">
+        <v>204</v>
+      </c>
+      <c r="B13" s="23">
+        <v>8.0</v>
+      </c>
+      <c r="C13" s="33">
+        <f t="shared" si="1"/>
+        <v>10</v>
+      </c>
+      <c r="D13" s="23" t="s">
+        <v>205</v>
+      </c>
+      <c r="E13" s="23">
+        <v>46.0</v>
+      </c>
+      <c r="F13" s="23">
+        <v>4.0</v>
+      </c>
+      <c r="G13" s="23">
+        <v>14.0</v>
+      </c>
+      <c r="H13" s="23" t="s">
+        <v>220</v>
+      </c>
+      <c r="I13" s="23" t="s">
+        <v>221</v>
+      </c>
+      <c r="J13" s="23" t="s">
+        <v>332</v>
+      </c>
+      <c r="K13" s="23" t="s">
+        <v>333</v>
+      </c>
+      <c r="L13" s="23" t="s">
+        <v>334</v>
+      </c>
+      <c r="M13" s="23" t="s">
+        <v>335</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="23" t="s">
+        <v>258</v>
+      </c>
+      <c r="B14" s="23">
+        <v>7.0</v>
+      </c>
+      <c r="C14" s="33">
+        <f t="shared" si="1"/>
+        <v>8.75</v>
+      </c>
+      <c r="D14" s="23" t="s">
+        <v>213</v>
+      </c>
+      <c r="E14" s="23">
+        <v>99.0</v>
+      </c>
+      <c r="F14" s="23">
+        <v>4.0</v>
+      </c>
+      <c r="G14" s="23">
+        <v>14.0</v>
+      </c>
+      <c r="H14" s="23" t="s">
+        <v>220</v>
+      </c>
+      <c r="I14" s="23" t="s">
+        <v>221</v>
+      </c>
+      <c r="J14" s="23" t="s">
+        <v>336</v>
+      </c>
+      <c r="K14" s="23" t="s">
+        <v>337</v>
+      </c>
+      <c r="L14" s="23" t="s">
+        <v>338</v>
+      </c>
+      <c r="M14" s="23" t="s">
+        <v>339</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="23" t="s">
+        <v>218</v>
+      </c>
+      <c r="B15" s="23">
         <v>6.0</v>
       </c>
-      <c r="G7" s="31">
-        <v>62.0</v>
-      </c>
-      <c r="H7" s="31" t="s">
-        <v>179</v>
-      </c>
-      <c r="I7" s="31" t="s">
-        <v>180</v>
-      </c>
-      <c r="J7" s="31" t="s">
-        <v>112</v>
-      </c>
-      <c r="K7" s="31" t="s">
-        <v>113</v>
-      </c>
-      <c r="L7" s="31" t="s">
-        <v>306</v>
-      </c>
-      <c r="M7" s="31" t="s">
-        <v>307</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="31" t="s">
-        <v>169</v>
-      </c>
-      <c r="B8" s="31">
-        <v>18.0</v>
-      </c>
-      <c r="C8" s="31">
-        <v>23.0</v>
-      </c>
-      <c r="D8" s="31" t="s">
-        <v>170</v>
-      </c>
-      <c r="E8" s="31">
-        <v>41.0</v>
-      </c>
-      <c r="F8" s="31">
-        <v>5.0</v>
-      </c>
-      <c r="G8" s="31">
-        <v>30.0</v>
-      </c>
-      <c r="H8" s="31" t="s">
-        <v>205</v>
-      </c>
-      <c r="I8" s="31" t="s">
-        <v>206</v>
-      </c>
-      <c r="J8" s="31" t="s">
-        <v>308</v>
-      </c>
-      <c r="K8" s="31" t="s">
-        <v>309</v>
-      </c>
-      <c r="L8" s="31" t="s">
-        <v>310</v>
-      </c>
-      <c r="M8" s="31" t="s">
-        <v>311</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="31" t="s">
-        <v>177</v>
-      </c>
-      <c r="B9" s="31">
-        <v>10.0</v>
-      </c>
-      <c r="C9" s="31">
-        <v>13.0</v>
-      </c>
-      <c r="D9" s="31" t="s">
-        <v>178</v>
-      </c>
-      <c r="E9" s="31">
-        <v>42.0</v>
-      </c>
-      <c r="F9" s="31">
+      <c r="C15" s="33">
+        <f t="shared" si="1"/>
+        <v>7.5</v>
+      </c>
+      <c r="D15" s="23" t="s">
+        <v>219</v>
+      </c>
+      <c r="E15" s="23">
+        <v>47.0</v>
+      </c>
+      <c r="F15" s="23">
         <v>4.0</v>
       </c>
-      <c r="G9" s="31">
+      <c r="G15" s="23">
         <v>14.0</v>
       </c>
-      <c r="H9" s="31" t="s">
-        <v>219</v>
-      </c>
-      <c r="I9" s="31" t="s">
+      <c r="H15" s="23" t="s">
         <v>220</v>
       </c>
-      <c r="J9" s="31" t="s">
-        <v>312</v>
-      </c>
-      <c r="K9" s="31" t="s">
-        <v>313</v>
-      </c>
-      <c r="L9" s="31" t="s">
-        <v>314</v>
-      </c>
-      <c r="M9" s="31" t="s">
-        <v>315</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="31" t="s">
-        <v>185</v>
-      </c>
-      <c r="B10" s="31">
-        <v>8.0</v>
-      </c>
-      <c r="C10" s="31">
-        <v>10.0</v>
-      </c>
-      <c r="D10" s="31" t="s">
-        <v>186</v>
-      </c>
-      <c r="E10" s="31">
-        <v>43.0</v>
-      </c>
-      <c r="F10" s="31">
-        <v>4.0</v>
-      </c>
-      <c r="G10" s="31">
-        <v>14.0</v>
-      </c>
-      <c r="H10" s="31" t="s">
-        <v>219</v>
-      </c>
-      <c r="I10" s="31" t="s">
-        <v>220</v>
-      </c>
-      <c r="J10" s="31" t="s">
-        <v>316</v>
-      </c>
-      <c r="K10" s="31" t="s">
-        <v>317</v>
-      </c>
-      <c r="L10" s="31" t="s">
-        <v>318</v>
-      </c>
-      <c r="M10" s="31" t="s">
-        <v>319</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="31" t="s">
-        <v>191</v>
-      </c>
-      <c r="B11" s="31">
-        <v>7.0</v>
-      </c>
-      <c r="C11" s="31">
-        <v>9.0</v>
-      </c>
-      <c r="D11" s="31" t="s">
-        <v>192</v>
-      </c>
-      <c r="E11" s="31">
-        <v>44.0</v>
-      </c>
-      <c r="F11" s="31">
-        <v>4.0</v>
-      </c>
-      <c r="G11" s="31">
-        <v>14.0</v>
-      </c>
-      <c r="H11" s="31" t="s">
-        <v>219</v>
-      </c>
-      <c r="I11" s="31" t="s">
-        <v>220</v>
-      </c>
-      <c r="J11" s="31" t="s">
-        <v>320</v>
-      </c>
-      <c r="K11" s="31" t="s">
-        <v>321</v>
-      </c>
-      <c r="L11" s="31" t="s">
-        <v>322</v>
-      </c>
-      <c r="M11" s="31" t="s">
-        <v>323</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="31" t="s">
-        <v>197</v>
-      </c>
-      <c r="B12" s="31">
-        <v>6.0</v>
-      </c>
-      <c r="C12" s="31">
-        <v>8.0</v>
-      </c>
-      <c r="D12" s="31" t="s">
-        <v>198</v>
-      </c>
-      <c r="E12" s="31">
-        <v>45.0</v>
-      </c>
-      <c r="F12" s="31">
-        <v>4.0</v>
-      </c>
-      <c r="G12" s="31">
-        <v>14.0</v>
-      </c>
-      <c r="H12" s="31" t="s">
-        <v>219</v>
-      </c>
-      <c r="I12" s="31" t="s">
-        <v>220</v>
-      </c>
-      <c r="J12" s="31" t="s">
-        <v>324</v>
-      </c>
-      <c r="K12" s="31" t="s">
-        <v>325</v>
-      </c>
-      <c r="L12" s="31" t="s">
-        <v>326</v>
-      </c>
-      <c r="M12" s="31" t="s">
-        <v>327</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="31" t="s">
-        <v>203</v>
-      </c>
-      <c r="B13" s="31">
-        <v>5.0</v>
-      </c>
-      <c r="C13" s="31">
-        <v>7.0</v>
-      </c>
-      <c r="D13" s="31" t="s">
-        <v>204</v>
-      </c>
-      <c r="E13" s="31">
-        <v>46.0</v>
-      </c>
-      <c r="F13" s="31">
-        <v>4.0</v>
-      </c>
-      <c r="G13" s="31">
-        <v>14.0</v>
-      </c>
-      <c r="H13" s="31" t="s">
-        <v>219</v>
-      </c>
-      <c r="I13" s="31" t="s">
-        <v>220</v>
-      </c>
-      <c r="J13" s="31" t="s">
-        <v>328</v>
-      </c>
-      <c r="K13" s="31" t="s">
-        <v>329</v>
-      </c>
-      <c r="L13" s="31" t="s">
-        <v>330</v>
-      </c>
-      <c r="M13" s="31" t="s">
-        <v>331</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="31" t="s">
-        <v>211</v>
-      </c>
-      <c r="B14" s="31">
-        <v>4.0</v>
-      </c>
-      <c r="C14" s="31">
-        <v>5.0</v>
-      </c>
-      <c r="D14" s="31" t="s">
-        <v>212</v>
-      </c>
-      <c r="E14" s="31">
-        <v>99.0</v>
-      </c>
-      <c r="F14" s="31">
-        <v>3.0</v>
-      </c>
-      <c r="G14" s="31">
-        <v>6.0</v>
-      </c>
-      <c r="H14" s="31" t="s">
-        <v>255</v>
-      </c>
-      <c r="I14" s="31" t="s">
-        <v>256</v>
-      </c>
-      <c r="J14" s="31" t="s">
-        <v>332</v>
-      </c>
-      <c r="K14" s="31" t="s">
-        <v>333</v>
-      </c>
-      <c r="L14" s="31" t="s">
-        <v>334</v>
-      </c>
-      <c r="M14" s="31" t="s">
-        <v>335</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="31" t="s">
-        <v>217</v>
-      </c>
-      <c r="B15" s="31">
-        <v>3.0</v>
-      </c>
-      <c r="C15" s="31">
-        <v>4.0</v>
-      </c>
-      <c r="D15" s="31" t="s">
-        <v>218</v>
-      </c>
-      <c r="E15" s="31">
-        <v>47.0</v>
-      </c>
-      <c r="F15" s="31">
-        <v>3.0</v>
-      </c>
-      <c r="G15" s="31">
-        <v>6.0</v>
-      </c>
-      <c r="H15" s="31" t="s">
-        <v>255</v>
-      </c>
-      <c r="I15" s="31" t="s">
-        <v>256</v>
-      </c>
-      <c r="J15" s="31" t="s">
-        <v>336</v>
-      </c>
-      <c r="K15" s="31" t="s">
-        <v>337</v>
-      </c>
-      <c r="L15" s="31" t="s">
-        <v>338</v>
-      </c>
-      <c r="M15" s="31" t="s">
-        <v>339</v>
+      <c r="I15" s="23" t="s">
+        <v>221</v>
+      </c>
+      <c r="J15" s="23" t="s">
+        <v>340</v>
+      </c>
+      <c r="K15" s="23" t="s">
+        <v>341</v>
+      </c>
+      <c r="L15" s="23" t="s">
+        <v>342</v>
+      </c>
+      <c r="M15" s="23" t="s">
+        <v>343</v>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="25" t="s">
-        <v>225</v>
-      </c>
-      <c r="B16" s="32">
+      <c r="A16" s="24" t="s">
+        <v>269</v>
+      </c>
+      <c r="B16" s="29">
         <v>96.0</v>
       </c>
-      <c r="C16" s="32">
+      <c r="C16" s="29">
         <v>123.0</v>
       </c>
       <c r="D16" s="28"/>
       <c r="E16" s="28"/>
       <c r="F16" s="28"/>
-      <c r="G16" s="32">
+      <c r="G16" s="29">
         <v>174.0</v>
       </c>
       <c r="H16" s="28"/>
@@ -7284,15 +7316,15 @@
       <c r="M17" s="28"/>
     </row>
     <row r="18">
-      <c r="A18" s="25" t="s">
-        <v>265</v>
-      </c>
-      <c r="B18" s="29" t="s">
-        <v>340</v>
-      </c>
-      <c r="C18" s="28"/>
-      <c r="D18" s="28"/>
-      <c r="E18" s="28"/>
+      <c r="A18" s="24" t="s">
+        <v>228</v>
+      </c>
+      <c r="B18" s="34" t="s">
+        <v>344</v>
+      </c>
+      <c r="C18" s="35"/>
+      <c r="D18" s="35"/>
+      <c r="E18" s="18"/>
       <c r="F18" s="28"/>
       <c r="G18" s="28"/>
       <c r="H18" s="28"/>
@@ -7319,7 +7351,7 @@
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="B1:D1"/>
+    <mergeCell ref="B18:E18"/>
   </mergeCells>
   <drawing r:id="rId1"/>
 </worksheet>
@@ -7334,7 +7366,7 @@
   <cols>
     <col customWidth="1" min="1" max="1" width="28.88"/>
     <col customWidth="1" min="6" max="6" width="14.25"/>
-    <col customWidth="1" min="7" max="7" width="15.5"/>
+    <col customWidth="1" min="7" max="7" width="17.13"/>
     <col customWidth="1" min="9" max="10" width="16.88"/>
     <col customWidth="1" min="11" max="11" width="17.13"/>
     <col customWidth="1" min="12" max="12" width="16.88"/>
@@ -7342,14 +7374,14 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="25" t="s">
+      <c r="A1" s="24" t="s">
         <v>150</v>
       </c>
-      <c r="B1" s="26" t="s">
-        <v>341</v>
-      </c>
-      <c r="C1" s="27"/>
-      <c r="D1" s="18"/>
+      <c r="B1" s="25" t="s">
+        <v>345</v>
+      </c>
+      <c r="C1" s="26"/>
+      <c r="D1" s="27"/>
       <c r="E1" s="28"/>
       <c r="F1" s="28"/>
       <c r="G1" s="28"/>
@@ -7362,10 +7394,10 @@
       <c r="N1" s="28"/>
     </row>
     <row r="2">
-      <c r="A2" s="25" t="s">
+      <c r="A2" s="24" t="s">
         <v>77</v>
       </c>
-      <c r="B2" s="29" t="s">
+      <c r="B2" s="25" t="s">
         <v>122</v>
       </c>
       <c r="C2" s="28"/>
@@ -7382,11 +7414,11 @@
       <c r="N2" s="28"/>
     </row>
     <row r="3">
-      <c r="A3" s="25" t="s">
+      <c r="A3" s="24" t="s">
         <v>79</v>
       </c>
-      <c r="B3" s="29" t="s">
-        <v>342</v>
+      <c r="B3" s="25" t="s">
+        <v>346</v>
       </c>
       <c r="C3" s="28"/>
       <c r="D3" s="28"/>
@@ -7434,439 +7466,439 @@
       <c r="N5" s="28"/>
     </row>
     <row r="6">
-      <c r="A6" s="30" t="s">
+      <c r="A6" s="36" t="s">
         <v>155</v>
       </c>
-      <c r="B6" s="30" t="s">
+      <c r="B6" s="36" t="s">
         <v>156</v>
       </c>
-      <c r="C6" s="30" t="s">
+      <c r="C6" s="36" t="s">
         <v>157</v>
       </c>
-      <c r="D6" s="30" t="s">
+      <c r="D6" s="36" t="s">
         <v>158</v>
       </c>
-      <c r="E6" s="30" t="s">
+      <c r="E6" s="36" t="s">
         <v>159</v>
       </c>
-      <c r="F6" s="30" t="s">
+      <c r="F6" s="36" t="s">
         <v>160</v>
       </c>
-      <c r="G6" s="30" t="s">
+      <c r="G6" s="36" t="s">
         <v>161</v>
       </c>
-      <c r="H6" s="30" t="s">
+      <c r="H6" s="36" t="s">
         <v>14</v>
       </c>
-      <c r="I6" s="30" t="s">
+      <c r="I6" s="36" t="s">
         <v>162</v>
       </c>
-      <c r="J6" s="30" t="s">
+      <c r="J6" s="36" t="s">
         <v>127</v>
       </c>
-      <c r="K6" s="30" t="s">
+      <c r="K6" s="36" t="s">
         <v>15</v>
       </c>
-      <c r="L6" s="30" t="s">
+      <c r="L6" s="36" t="s">
         <v>16</v>
       </c>
-      <c r="M6" s="30" t="s">
-        <v>228</v>
+      <c r="M6" s="36" t="s">
+        <v>163</v>
       </c>
       <c r="N6" s="28"/>
     </row>
     <row r="7">
-      <c r="A7" s="31" t="s">
-        <v>163</v>
-      </c>
-      <c r="B7" s="31">
+      <c r="A7" s="23" t="s">
+        <v>164</v>
+      </c>
+      <c r="B7" s="23">
         <v>36.0</v>
       </c>
-      <c r="C7" s="31">
+      <c r="C7" s="23">
         <v>45.0</v>
       </c>
-      <c r="D7" s="31" t="s">
-        <v>164</v>
-      </c>
-      <c r="E7" s="31">
+      <c r="D7" s="23" t="s">
+        <v>165</v>
+      </c>
+      <c r="E7" s="23">
         <v>30.0</v>
       </c>
-      <c r="F7" s="31">
+      <c r="F7" s="23">
         <v>6.0</v>
       </c>
-      <c r="G7" s="31">
+      <c r="G7" s="23">
         <v>62.0</v>
       </c>
-      <c r="H7" s="31" t="s">
+      <c r="H7" s="23" t="s">
+        <v>180</v>
+      </c>
+      <c r="I7" s="23" t="s">
+        <v>181</v>
+      </c>
+      <c r="J7" s="23" t="s">
+        <v>118</v>
+      </c>
+      <c r="K7" s="23" t="s">
+        <v>119</v>
+      </c>
+      <c r="L7" s="23" t="s">
+        <v>347</v>
+      </c>
+      <c r="M7" s="23" t="s">
+        <v>348</v>
+      </c>
+      <c r="N7" s="28"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="23" t="s">
+        <v>170</v>
+      </c>
+      <c r="B8" s="23">
+        <v>20.0</v>
+      </c>
+      <c r="C8" s="23">
+        <v>25.0</v>
+      </c>
+      <c r="D8" s="23" t="s">
+        <v>171</v>
+      </c>
+      <c r="E8" s="23">
+        <v>10.0</v>
+      </c>
+      <c r="F8" s="23">
+        <v>5.0</v>
+      </c>
+      <c r="G8" s="23">
+        <v>30.0</v>
+      </c>
+      <c r="H8" s="23" t="s">
+        <v>206</v>
+      </c>
+      <c r="I8" s="23" t="s">
+        <v>207</v>
+      </c>
+      <c r="J8" s="23" t="s">
+        <v>349</v>
+      </c>
+      <c r="K8" s="23" t="s">
+        <v>350</v>
+      </c>
+      <c r="L8" s="23" t="s">
+        <v>351</v>
+      </c>
+      <c r="M8" s="23" t="s">
+        <v>352</v>
+      </c>
+      <c r="N8" s="28"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="23" t="s">
+        <v>178</v>
+      </c>
+      <c r="B9" s="23">
+        <v>11.0</v>
+      </c>
+      <c r="C9" s="23">
+        <v>14.0</v>
+      </c>
+      <c r="D9" s="23" t="s">
         <v>179</v>
       </c>
-      <c r="I7" s="31" t="s">
-        <v>180</v>
-      </c>
-      <c r="J7" s="31" t="s">
-        <v>118</v>
-      </c>
-      <c r="K7" s="31" t="s">
-        <v>119</v>
-      </c>
-      <c r="L7" s="31" t="s">
-        <v>343</v>
-      </c>
-      <c r="M7" s="31" t="s">
-        <v>344</v>
-      </c>
-      <c r="N7" s="28"/>
-    </row>
-    <row r="8">
-      <c r="A8" s="31" t="s">
-        <v>169</v>
-      </c>
-      <c r="B8" s="31">
+      <c r="E9" s="23">
+        <v>40.0</v>
+      </c>
+      <c r="F9" s="23">
+        <v>4.0</v>
+      </c>
+      <c r="G9" s="23">
+        <v>14.0</v>
+      </c>
+      <c r="H9" s="23" t="s">
+        <v>220</v>
+      </c>
+      <c r="I9" s="23" t="s">
+        <v>221</v>
+      </c>
+      <c r="J9" s="23" t="s">
+        <v>353</v>
+      </c>
+      <c r="K9" s="23" t="s">
+        <v>354</v>
+      </c>
+      <c r="L9" s="23" t="s">
+        <v>355</v>
+      </c>
+      <c r="M9" s="23" t="s">
+        <v>356</v>
+      </c>
+      <c r="N9" s="28"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="23" t="s">
+        <v>186</v>
+      </c>
+      <c r="B10" s="23">
+        <v>9.0</v>
+      </c>
+      <c r="C10" s="23">
+        <v>12.0</v>
+      </c>
+      <c r="D10" s="23" t="s">
+        <v>187</v>
+      </c>
+      <c r="E10" s="23">
+        <v>80.0</v>
+      </c>
+      <c r="F10" s="23">
+        <v>4.0</v>
+      </c>
+      <c r="G10" s="23">
+        <v>14.0</v>
+      </c>
+      <c r="H10" s="23" t="s">
+        <v>220</v>
+      </c>
+      <c r="I10" s="23" t="s">
+        <v>221</v>
+      </c>
+      <c r="J10" s="23" t="s">
+        <v>357</v>
+      </c>
+      <c r="K10" s="23" t="s">
+        <v>358</v>
+      </c>
+      <c r="L10" s="23" t="s">
+        <v>359</v>
+      </c>
+      <c r="M10" s="23" t="s">
+        <v>360</v>
+      </c>
+      <c r="N10" s="28"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="23" t="s">
+        <v>192</v>
+      </c>
+      <c r="B11" s="23">
+        <v>8.0</v>
+      </c>
+      <c r="C11" s="23">
+        <v>10.0</v>
+      </c>
+      <c r="D11" s="23" t="s">
+        <v>193</v>
+      </c>
+      <c r="E11" s="23">
+        <v>50.0</v>
+      </c>
+      <c r="F11" s="23">
+        <v>4.0</v>
+      </c>
+      <c r="G11" s="23">
+        <v>14.0</v>
+      </c>
+      <c r="H11" s="23" t="s">
+        <v>220</v>
+      </c>
+      <c r="I11" s="23" t="s">
+        <v>221</v>
+      </c>
+      <c r="J11" s="23" t="s">
+        <v>361</v>
+      </c>
+      <c r="K11" s="23" t="s">
+        <v>362</v>
+      </c>
+      <c r="L11" s="23" t="s">
+        <v>363</v>
+      </c>
+      <c r="M11" s="23" t="s">
+        <v>364</v>
+      </c>
+      <c r="N11" s="28"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="23" t="s">
+        <v>198</v>
+      </c>
+      <c r="B12" s="23">
+        <v>7.0</v>
+      </c>
+      <c r="C12" s="23">
+        <v>9.0</v>
+      </c>
+      <c r="D12" s="23" t="s">
+        <v>199</v>
+      </c>
+      <c r="E12" s="23">
         <v>20.0</v>
       </c>
-      <c r="C8" s="31">
-        <v>25.0</v>
-      </c>
-      <c r="D8" s="31" t="s">
-        <v>170</v>
-      </c>
-      <c r="E8" s="31">
-        <v>10.0</v>
-      </c>
-      <c r="F8" s="31">
+      <c r="F12" s="23">
+        <v>4.0</v>
+      </c>
+      <c r="G12" s="23">
+        <v>14.0</v>
+      </c>
+      <c r="H12" s="23" t="s">
+        <v>220</v>
+      </c>
+      <c r="I12" s="23" t="s">
+        <v>221</v>
+      </c>
+      <c r="J12" s="23" t="s">
+        <v>365</v>
+      </c>
+      <c r="K12" s="23" t="s">
+        <v>366</v>
+      </c>
+      <c r="L12" s="23" t="s">
+        <v>367</v>
+      </c>
+      <c r="M12" s="23" t="s">
+        <v>368</v>
+      </c>
+      <c r="N12" s="28"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="23" t="s">
+        <v>204</v>
+      </c>
+      <c r="B13" s="23">
         <v>5.0</v>
       </c>
-      <c r="G8" s="31">
-        <v>30.0</v>
-      </c>
-      <c r="H8" s="31" t="s">
+      <c r="C13" s="23">
+        <v>7.0</v>
+      </c>
+      <c r="D13" s="23" t="s">
         <v>205</v>
       </c>
-      <c r="I8" s="31" t="s">
-        <v>206</v>
-      </c>
-      <c r="J8" s="31" t="s">
-        <v>345</v>
-      </c>
-      <c r="K8" s="31" t="s">
-        <v>346</v>
-      </c>
-      <c r="L8" s="31" t="s">
-        <v>347</v>
-      </c>
-      <c r="M8" s="31" t="s">
-        <v>348</v>
-      </c>
-      <c r="N8" s="28"/>
-    </row>
-    <row r="9">
-      <c r="A9" s="31" t="s">
-        <v>177</v>
-      </c>
-      <c r="B9" s="31">
-        <v>11.0</v>
-      </c>
-      <c r="C9" s="31">
+      <c r="E13" s="23">
+        <v>70.0</v>
+      </c>
+      <c r="F13" s="23">
+        <v>4.0</v>
+      </c>
+      <c r="G13" s="23">
         <v>14.0</v>
       </c>
-      <c r="D9" s="31" t="s">
-        <v>178</v>
-      </c>
-      <c r="E9" s="31">
-        <v>40.0</v>
-      </c>
-      <c r="F9" s="31">
+      <c r="H13" s="23" t="s">
+        <v>220</v>
+      </c>
+      <c r="I13" s="23" t="s">
+        <v>221</v>
+      </c>
+      <c r="J13" s="23" t="s">
+        <v>369</v>
+      </c>
+      <c r="K13" s="23" t="s">
+        <v>370</v>
+      </c>
+      <c r="L13" s="23" t="s">
+        <v>371</v>
+      </c>
+      <c r="M13" s="23" t="s">
+        <v>372</v>
+      </c>
+      <c r="N13" s="28"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="23" t="s">
+        <v>218</v>
+      </c>
+      <c r="B14" s="23">
+        <v>5.0</v>
+      </c>
+      <c r="C14" s="23">
+        <v>7.0</v>
+      </c>
+      <c r="D14" s="23" t="s">
+        <v>219</v>
+      </c>
+      <c r="E14" s="23">
+        <v>60.0</v>
+      </c>
+      <c r="F14" s="23">
         <v>4.0</v>
       </c>
-      <c r="G9" s="31">
+      <c r="G14" s="23">
         <v>14.0</v>
       </c>
-      <c r="H9" s="31" t="s">
-        <v>219</v>
-      </c>
-      <c r="I9" s="31" t="s">
+      <c r="H14" s="23" t="s">
         <v>220</v>
       </c>
-      <c r="J9" s="31" t="s">
-        <v>349</v>
-      </c>
-      <c r="K9" s="31" t="s">
-        <v>350</v>
-      </c>
-      <c r="L9" s="31" t="s">
-        <v>351</v>
-      </c>
-      <c r="M9" s="31" t="s">
-        <v>352</v>
-      </c>
-      <c r="N9" s="28"/>
-    </row>
-    <row r="10">
-      <c r="A10" s="31" t="s">
-        <v>185</v>
-      </c>
-      <c r="B10" s="31">
-        <v>9.0</v>
-      </c>
-      <c r="C10" s="31">
-        <v>12.0</v>
-      </c>
-      <c r="D10" s="31" t="s">
-        <v>186</v>
-      </c>
-      <c r="E10" s="31">
-        <v>80.0</v>
-      </c>
-      <c r="F10" s="31">
+      <c r="I14" s="23" t="s">
+        <v>221</v>
+      </c>
+      <c r="J14" s="23" t="s">
+        <v>373</v>
+      </c>
+      <c r="K14" s="23" t="s">
+        <v>374</v>
+      </c>
+      <c r="L14" s="23" t="s">
+        <v>375</v>
+      </c>
+      <c r="M14" s="23" t="s">
+        <v>376</v>
+      </c>
+      <c r="N14" s="28"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="23" t="s">
+        <v>258</v>
+      </c>
+      <c r="B15" s="23">
         <v>4.0</v>
       </c>
-      <c r="G10" s="31">
-        <v>14.0</v>
-      </c>
-      <c r="H10" s="31" t="s">
-        <v>219</v>
-      </c>
-      <c r="I10" s="31" t="s">
-        <v>220</v>
-      </c>
-      <c r="J10" s="31" t="s">
-        <v>353</v>
-      </c>
-      <c r="K10" s="31" t="s">
-        <v>354</v>
-      </c>
-      <c r="L10" s="31" t="s">
-        <v>355</v>
-      </c>
-      <c r="M10" s="31" t="s">
-        <v>356</v>
-      </c>
-      <c r="N10" s="28"/>
-    </row>
-    <row r="11">
-      <c r="A11" s="31" t="s">
-        <v>191</v>
-      </c>
-      <c r="B11" s="31">
-        <v>8.0</v>
-      </c>
-      <c r="C11" s="31">
-        <v>10.0</v>
-      </c>
-      <c r="D11" s="31" t="s">
-        <v>192</v>
-      </c>
-      <c r="E11" s="31">
-        <v>50.0</v>
-      </c>
-      <c r="F11" s="31">
-        <v>4.0</v>
-      </c>
-      <c r="G11" s="31">
-        <v>14.0</v>
-      </c>
-      <c r="H11" s="31" t="s">
-        <v>219</v>
-      </c>
-      <c r="I11" s="31" t="s">
-        <v>220</v>
-      </c>
-      <c r="J11" s="31" t="s">
-        <v>357</v>
-      </c>
-      <c r="K11" s="31" t="s">
-        <v>358</v>
-      </c>
-      <c r="L11" s="31" t="s">
-        <v>359</v>
-      </c>
-      <c r="M11" s="31" t="s">
-        <v>360</v>
-      </c>
-      <c r="N11" s="28"/>
-    </row>
-    <row r="12">
-      <c r="A12" s="31" t="s">
-        <v>197</v>
-      </c>
-      <c r="B12" s="31">
-        <v>7.0</v>
-      </c>
-      <c r="C12" s="31">
-        <v>9.0</v>
-      </c>
-      <c r="D12" s="31" t="s">
-        <v>198</v>
-      </c>
-      <c r="E12" s="31">
-        <v>20.0</v>
-      </c>
-      <c r="F12" s="31">
-        <v>4.0</v>
-      </c>
-      <c r="G12" s="31">
-        <v>14.0</v>
-      </c>
-      <c r="H12" s="31" t="s">
-        <v>219</v>
-      </c>
-      <c r="I12" s="31" t="s">
-        <v>220</v>
-      </c>
-      <c r="J12" s="31" t="s">
-        <v>361</v>
-      </c>
-      <c r="K12" s="31" t="s">
-        <v>362</v>
-      </c>
-      <c r="L12" s="31" t="s">
-        <v>363</v>
-      </c>
-      <c r="M12" s="31" t="s">
-        <v>364</v>
-      </c>
-      <c r="N12" s="28"/>
-    </row>
-    <row r="13">
-      <c r="A13" s="31" t="s">
-        <v>203</v>
-      </c>
-      <c r="B13" s="31">
+      <c r="C15" s="23">
         <v>5.0</v>
       </c>
-      <c r="C13" s="31">
-        <v>7.0</v>
-      </c>
-      <c r="D13" s="31" t="s">
-        <v>204</v>
-      </c>
-      <c r="E13" s="31">
-        <v>70.0</v>
-      </c>
-      <c r="F13" s="31">
-        <v>4.0</v>
-      </c>
-      <c r="G13" s="31">
-        <v>14.0</v>
-      </c>
-      <c r="H13" s="31" t="s">
-        <v>219</v>
-      </c>
-      <c r="I13" s="31" t="s">
-        <v>220</v>
-      </c>
-      <c r="J13" s="31" t="s">
-        <v>365</v>
-      </c>
-      <c r="K13" s="31" t="s">
-        <v>366</v>
-      </c>
-      <c r="L13" s="31" t="s">
-        <v>367</v>
-      </c>
-      <c r="M13" s="31" t="s">
-        <v>368</v>
-      </c>
-      <c r="N13" s="28"/>
-    </row>
-    <row r="14">
-      <c r="A14" s="31" t="s">
-        <v>217</v>
-      </c>
-      <c r="B14" s="31">
-        <v>5.0</v>
-      </c>
-      <c r="C14" s="31">
-        <v>7.0</v>
-      </c>
-      <c r="D14" s="31" t="s">
-        <v>218</v>
-      </c>
-      <c r="E14" s="31">
-        <v>60.0</v>
-      </c>
-      <c r="F14" s="31">
-        <v>4.0</v>
-      </c>
-      <c r="G14" s="31">
-        <v>14.0</v>
-      </c>
-      <c r="H14" s="31" t="s">
-        <v>219</v>
-      </c>
-      <c r="I14" s="31" t="s">
-        <v>220</v>
-      </c>
-      <c r="J14" s="31" t="s">
-        <v>369</v>
-      </c>
-      <c r="K14" s="31" t="s">
-        <v>370</v>
-      </c>
-      <c r="L14" s="31" t="s">
-        <v>371</v>
-      </c>
-      <c r="M14" s="31" t="s">
-        <v>372</v>
-      </c>
-      <c r="N14" s="28"/>
-    </row>
-    <row r="15">
-      <c r="A15" s="31" t="s">
-        <v>211</v>
-      </c>
-      <c r="B15" s="31">
-        <v>4.0</v>
-      </c>
-      <c r="C15" s="31">
-        <v>5.0</v>
-      </c>
-      <c r="D15" s="31" t="s">
-        <v>212</v>
-      </c>
-      <c r="E15" s="31">
+      <c r="D15" s="23" t="s">
+        <v>213</v>
+      </c>
+      <c r="E15" s="23">
         <v>99.0</v>
       </c>
-      <c r="F15" s="31">
+      <c r="F15" s="23">
         <v>3.0</v>
       </c>
-      <c r="G15" s="31">
+      <c r="G15" s="23">
         <v>6.0</v>
       </c>
-      <c r="H15" s="31" t="s">
-        <v>255</v>
-      </c>
-      <c r="I15" s="31" t="s">
-        <v>256</v>
-      </c>
-      <c r="J15" s="31" t="s">
-        <v>373</v>
-      </c>
-      <c r="K15" s="31" t="s">
-        <v>374</v>
-      </c>
-      <c r="L15" s="31" t="s">
-        <v>375</v>
-      </c>
-      <c r="M15" s="31" t="s">
-        <v>376</v>
+      <c r="H15" s="23" t="s">
+        <v>259</v>
+      </c>
+      <c r="I15" s="23" t="s">
+        <v>260</v>
+      </c>
+      <c r="J15" s="23" t="s">
+        <v>377</v>
+      </c>
+      <c r="K15" s="23" t="s">
+        <v>378</v>
+      </c>
+      <c r="L15" s="23" t="s">
+        <v>379</v>
+      </c>
+      <c r="M15" s="23" t="s">
+        <v>380</v>
       </c>
       <c r="N15" s="28"/>
     </row>
     <row r="16">
-      <c r="A16" s="25" t="s">
-        <v>225</v>
-      </c>
-      <c r="B16" s="32">
+      <c r="A16" s="24" t="s">
+        <v>269</v>
+      </c>
+      <c r="B16" s="29">
         <v>105.0</v>
       </c>
-      <c r="C16" s="32">
+      <c r="C16" s="29">
         <v>134.0</v>
       </c>
       <c r="D16" s="28"/>
       <c r="E16" s="28"/>
       <c r="F16" s="28"/>
-      <c r="G16" s="32">
+      <c r="G16" s="29">
         <v>182.0</v>
       </c>
       <c r="H16" s="28"/>
@@ -7894,11 +7926,11 @@
       <c r="N17" s="28"/>
     </row>
     <row r="18">
-      <c r="A18" s="25" t="s">
-        <v>265</v>
-      </c>
-      <c r="B18" s="29" t="s">
-        <v>377</v>
+      <c r="A18" s="24" t="s">
+        <v>228</v>
+      </c>
+      <c r="B18" s="25" t="s">
+        <v>381</v>
       </c>
       <c r="C18" s="28"/>
       <c r="D18" s="28"/>
@@ -7925,7 +7957,9 @@
       <c r="I19" s="28"/>
       <c r="J19" s="28"/>
       <c r="K19" s="28"/>
-      <c r="L19" s="28"/>
+      <c r="L19" s="23" t="s">
+        <v>382</v>
+      </c>
       <c r="M19" s="28"/>
       <c r="N19" s="28"/>
     </row>
@@ -7939,9 +7973,13 @@
       <c r="G20" s="28"/>
       <c r="H20" s="28"/>
       <c r="I20" s="28"/>
-      <c r="J20" s="28"/>
+      <c r="J20" s="23" t="s">
+        <v>358</v>
+      </c>
       <c r="K20" s="28"/>
-      <c r="L20" s="28"/>
+      <c r="L20" s="23" t="s">
+        <v>383</v>
+      </c>
       <c r="M20" s="28"/>
       <c r="N20" s="28"/>
     </row>
@@ -8026,9 +8064,6 @@
       <c r="N25" s="28"/>
     </row>
   </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="B1:D1"/>
-  </mergeCells>
   <drawing r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update DNS settings and IP addresses for various devices in Lima network configuration
</commit_message>
<xml_diff>
--- a/excel-final/Esquema de Direccionamiento IP.xlsx
+++ b/excel-final/Esquema de Direccionamiento IP.xlsx
@@ -655,16 +655,40 @@
     <t>10.192.42.159</t>
   </si>
   <si>
+    <t>Servidores</t>
+  </si>
+  <si>
+    <t>VLSER</t>
+  </si>
+  <si>
+    <t>/28</t>
+  </si>
+  <si>
+    <t>255.255.255.240</t>
+  </si>
+  <si>
+    <t>10.192.42.160</t>
+  </si>
+  <si>
+    <t>10.192.42.161</t>
+  </si>
+  <si>
+    <t>10.192.42.174</t>
+  </si>
+  <si>
+    <t>10.192.42.175</t>
+  </si>
+  <si>
     <t>Nativa</t>
   </si>
   <si>
     <t>VLNAT</t>
   </si>
   <si>
-    <t>10.192.42.160</t>
-  </si>
-  <si>
-    <t>10.192.42.161</t>
+    <t>10.192.42.176</t>
+  </si>
+  <si>
+    <t>10.192.42.177</t>
   </si>
   <si>
     <t>10.192.42.190</t>
@@ -673,34 +697,10 @@
     <t>10.192.42.191</t>
   </si>
   <si>
-    <t>Servidores</t>
-  </si>
-  <si>
-    <t>VLSER</t>
-  </si>
-  <si>
-    <t>/28</t>
-  </si>
-  <si>
-    <t>255.255.255.240</t>
-  </si>
-  <si>
-    <t>10.192.42.192</t>
-  </si>
-  <si>
-    <t>10.192.42.193</t>
-  </si>
-  <si>
-    <t>10.192.42.206</t>
-  </si>
-  <si>
-    <t>10.192.42.207</t>
-  </si>
-  <si>
     <t>Nota:</t>
   </si>
   <si>
-    <t>Los 452 hosts corresponden a los requerimientos indicados en el caso para Lima. Adicionalmente, se dimensionan 15 hosts para la VLAN Nativa/Gestión, de acuerdo con la cantidad de dispositivos de red considerados en la solución, obteniendo un total de 467 hosts dimensionados.</t>
+    <t>Los 452 hosts corresponden a los requerimientos indicados en el caso para Lima. Adicionalmente, se dimensionan 9 hosts actuales para la VLAN Nativa/Gestión según los dispositivos de red usados; con crecimiento del 25% se consideran 12 hosts. Total actual dimensionado: 461 hosts.</t>
   </si>
   <si>
     <t>Validacion:</t>
@@ -904,130 +904,130 @@
     <t>10.192.49.31</t>
   </si>
   <si>
+    <t>10.192.49.32</t>
+  </si>
+  <si>
+    <t>10.192.49.33</t>
+  </si>
+  <si>
+    <t>10.192.49.46</t>
+  </si>
+  <si>
+    <t>10.192.49.47</t>
+  </si>
+  <si>
+    <t>10.192.49.48</t>
+  </si>
+  <si>
+    <t>10.192.49.49</t>
+  </si>
+  <si>
+    <t>10.192.49.62</t>
+  </si>
+  <si>
+    <t>10.192.49.63</t>
+  </si>
+  <si>
+    <t>10.192.49.64</t>
+  </si>
+  <si>
+    <t>10.192.49.65</t>
+  </si>
+  <si>
+    <t>10.192.49.78</t>
+  </si>
+  <si>
+    <t>10.192.49.79</t>
+  </si>
+  <si>
+    <t>Todas las VLAN quedan dentro de 10.192.48.0/22 y no se solapan.</t>
+  </si>
+  <si>
+    <t>Portalanza Romero, Aurora de Libertad</t>
+  </si>
+  <si>
+    <t>10.192.52.0/22</t>
+  </si>
+  <si>
+    <t>10.192.52.30</t>
+  </si>
+  <si>
+    <t>10.192.52.31</t>
+  </si>
+  <si>
+    <t>10.192.52.32</t>
+  </si>
+  <si>
+    <t>10.192.52.33</t>
+  </si>
+  <si>
+    <t>10.192.52.62</t>
+  </si>
+  <si>
+    <t>10.192.52.63</t>
+  </si>
+  <si>
+    <t>10.192.52.64</t>
+  </si>
+  <si>
+    <t>10.192.52.65</t>
+  </si>
+  <si>
+    <t>10.192.52.94</t>
+  </si>
+  <si>
+    <t>10.192.52.95</t>
+  </si>
+  <si>
+    <t>10.192.52.96</t>
+  </si>
+  <si>
+    <t>10.192.52.97</t>
+  </si>
+  <si>
+    <t>10.192.52.110</t>
+  </si>
+  <si>
+    <t>10.192.52.111</t>
+  </si>
+  <si>
+    <t>10.192.52.112</t>
+  </si>
+  <si>
+    <t>10.192.52.113</t>
+  </si>
+  <si>
+    <t>10.192.52.126</t>
+  </si>
+  <si>
+    <t>10.192.52.127</t>
+  </si>
+  <si>
+    <t>10.192.52.128</t>
+  </si>
+  <si>
+    <t>10.192.52.129</t>
+  </si>
+  <si>
+    <t>10.192.52.142</t>
+  </si>
+  <si>
+    <t>10.192.52.143</t>
+  </si>
+  <si>
+    <t>10.192.52.144</t>
+  </si>
+  <si>
+    <t>10.192.52.145</t>
+  </si>
+  <si>
+    <t>10.192.52.158</t>
+  </si>
+  <si>
+    <t>10.192.52.159</t>
+  </si>
+  <si>
     <t>Nativa/Gestion</t>
-  </si>
-  <si>
-    <t>10.192.49.32</t>
-  </si>
-  <si>
-    <t>10.192.49.33</t>
-  </si>
-  <si>
-    <t>10.192.49.46</t>
-  </si>
-  <si>
-    <t>10.192.49.47</t>
-  </si>
-  <si>
-    <t>10.192.49.48</t>
-  </si>
-  <si>
-    <t>10.192.49.49</t>
-  </si>
-  <si>
-    <t>10.192.49.62</t>
-  </si>
-  <si>
-    <t>10.192.49.63</t>
-  </si>
-  <si>
-    <t>10.192.49.64</t>
-  </si>
-  <si>
-    <t>10.192.49.65</t>
-  </si>
-  <si>
-    <t>10.192.49.78</t>
-  </si>
-  <si>
-    <t>10.192.49.79</t>
-  </si>
-  <si>
-    <t>Todas las VLAN quedan dentro de 10.192.48.0/22 y no se solapan.</t>
-  </si>
-  <si>
-    <t>Portalanza Romero, Aurora de Libertad</t>
-  </si>
-  <si>
-    <t>10.192.52.0/22</t>
-  </si>
-  <si>
-    <t>10.192.52.30</t>
-  </si>
-  <si>
-    <t>10.192.52.31</t>
-  </si>
-  <si>
-    <t>10.192.52.32</t>
-  </si>
-  <si>
-    <t>10.192.52.33</t>
-  </si>
-  <si>
-    <t>10.192.52.62</t>
-  </si>
-  <si>
-    <t>10.192.52.63</t>
-  </si>
-  <si>
-    <t>10.192.52.64</t>
-  </si>
-  <si>
-    <t>10.192.52.65</t>
-  </si>
-  <si>
-    <t>10.192.52.94</t>
-  </si>
-  <si>
-    <t>10.192.52.95</t>
-  </si>
-  <si>
-    <t>10.192.52.96</t>
-  </si>
-  <si>
-    <t>10.192.52.97</t>
-  </si>
-  <si>
-    <t>10.192.52.110</t>
-  </si>
-  <si>
-    <t>10.192.52.111</t>
-  </si>
-  <si>
-    <t>10.192.52.112</t>
-  </si>
-  <si>
-    <t>10.192.52.113</t>
-  </si>
-  <si>
-    <t>10.192.52.126</t>
-  </si>
-  <si>
-    <t>10.192.52.127</t>
-  </si>
-  <si>
-    <t>10.192.52.128</t>
-  </si>
-  <si>
-    <t>10.192.52.129</t>
-  </si>
-  <si>
-    <t>10.192.52.142</t>
-  </si>
-  <si>
-    <t>10.192.52.143</t>
-  </si>
-  <si>
-    <t>10.192.52.144</t>
-  </si>
-  <si>
-    <t>10.192.52.145</t>
-  </si>
-  <si>
-    <t>10.192.52.158</t>
-  </si>
-  <si>
-    <t>10.192.52.159</t>
   </si>
   <si>
     <t>10.192.52.160</t>
@@ -1251,7 +1251,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="16">
+  <borders count="15">
     <border/>
     <border>
       <left style="thin">
@@ -1367,14 +1367,6 @@
       <right style="thin">
         <color rgb="FF000000"/>
       </right>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF000000"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF000000"/>
-      </right>
       <bottom style="thin">
         <color rgb="FF000000"/>
       </bottom>
@@ -1452,7 +1444,7 @@
       <alignment horizontal="center" readingOrder="0" shrinkToFit="0" wrapText="1"/>
     </xf>
     <xf borderId="1" fillId="0" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0" shrinkToFit="0" wrapText="0"/>
+      <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyFont="1"/>
     <xf borderId="1" fillId="0" fontId="9" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
@@ -1520,20 +1512,20 @@
     <xf borderId="1" fillId="4" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
+    <xf borderId="1" fillId="0" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0" shrinkToFit="0" wrapText="0"/>
+    </xf>
     <xf borderId="2" fillId="0" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
     <xf borderId="13" fillId="4" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0" shrinkToFit="0" wrapText="1"/>
     </xf>
-    <xf borderId="13" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0"/>
+    <xf borderId="14" fillId="0" fontId="9" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
-    <xf borderId="14" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0"/>
-    </xf>
-    <xf borderId="15" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0"/>
+    <xf borderId="14" fillId="0" fontId="9" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="right" readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -3117,57 +3109,57 @@
         <v>212</v>
       </c>
       <c r="B14" s="23">
-        <v>15.0</v>
+        <v>10.0</v>
       </c>
       <c r="C14" s="23">
-        <v>19.0</v>
+        <v>13.0</v>
       </c>
       <c r="D14" s="23" t="s">
         <v>213</v>
       </c>
       <c r="E14" s="23">
-        <v>99.0</v>
+        <v>17.0</v>
       </c>
       <c r="F14" s="23">
-        <v>5.0</v>
+        <v>4.0</v>
       </c>
       <c r="G14" s="23">
-        <v>30.0</v>
+        <v>14.0</v>
       </c>
       <c r="H14" s="23" t="s">
-        <v>206</v>
+        <v>214</v>
       </c>
       <c r="I14" s="23" t="s">
-        <v>207</v>
+        <v>215</v>
       </c>
       <c r="J14" s="23" t="s">
-        <v>214</v>
+        <v>216</v>
       </c>
       <c r="K14" s="23" t="s">
-        <v>215</v>
+        <v>217</v>
       </c>
       <c r="L14" s="23" t="s">
-        <v>216</v>
+        <v>218</v>
       </c>
       <c r="M14" s="23" t="s">
-        <v>217</v>
+        <v>219</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="23" t="s">
-        <v>218</v>
+        <v>220</v>
       </c>
       <c r="B15" s="23">
-        <v>10.0</v>
+        <v>9.0</v>
       </c>
       <c r="C15" s="23">
-        <v>13.0</v>
+        <v>12.0</v>
       </c>
       <c r="D15" s="23" t="s">
-        <v>219</v>
+        <v>221</v>
       </c>
       <c r="E15" s="23">
-        <v>17.0</v>
+        <v>99.0</v>
       </c>
       <c r="F15" s="23">
         <v>4.0</v>
@@ -3176,10 +3168,10 @@
         <v>14.0</v>
       </c>
       <c r="H15" s="23" t="s">
-        <v>220</v>
+        <v>214</v>
       </c>
       <c r="I15" s="23" t="s">
-        <v>221</v>
+        <v>215</v>
       </c>
       <c r="J15" s="23" t="s">
         <v>222</v>
@@ -3197,12 +3189,12 @@
     <row r="16">
       <c r="B16" s="24">
         <f>SUM(B7:B15)</f>
-        <v>467</v>
+        <v>461</v>
       </c>
     </row>
     <row r="17">
       <c r="B17" s="24">
-        <f>B16-15</f>
+        <f>B16-9</f>
         <v>452</v>
       </c>
     </row>
@@ -3541,10 +3533,10 @@
         <v>14.0</v>
       </c>
       <c r="H10" s="38" t="s">
-        <v>220</v>
+        <v>214</v>
       </c>
       <c r="I10" s="38" t="s">
-        <v>221</v>
+        <v>215</v>
       </c>
       <c r="J10" s="38" t="s">
         <v>243</v>
@@ -3582,10 +3574,10 @@
         <v>14.0</v>
       </c>
       <c r="H11" s="38" t="s">
-        <v>220</v>
+        <v>214</v>
       </c>
       <c r="I11" s="38" t="s">
-        <v>221</v>
+        <v>215</v>
       </c>
       <c r="J11" s="38" t="s">
         <v>247</v>
@@ -3623,10 +3615,10 @@
         <v>14.0</v>
       </c>
       <c r="H12" s="38" t="s">
-        <v>220</v>
+        <v>214</v>
       </c>
       <c r="I12" s="38" t="s">
-        <v>221</v>
+        <v>215</v>
       </c>
       <c r="J12" s="38" t="s">
         <v>252</v>
@@ -3652,7 +3644,7 @@
         <v>12.0</v>
       </c>
       <c r="D13" s="38" t="s">
-        <v>213</v>
+        <v>221</v>
       </c>
       <c r="E13" s="38">
         <v>99.0</v>
@@ -3664,10 +3656,10 @@
         <v>14.0</v>
       </c>
       <c r="H13" s="38" t="s">
-        <v>220</v>
+        <v>214</v>
       </c>
       <c r="I13" s="38" t="s">
-        <v>221</v>
+        <v>215</v>
       </c>
       <c r="J13" s="38" t="s">
         <v>257</v>
@@ -3705,10 +3697,10 @@
         <v>14.0</v>
       </c>
       <c r="H14" s="38" t="s">
-        <v>220</v>
+        <v>214</v>
       </c>
       <c r="I14" s="38" t="s">
-        <v>221</v>
+        <v>215</v>
       </c>
       <c r="J14" s="38" t="s">
         <v>261</v>
@@ -3725,7 +3717,7 @@
     </row>
     <row r="15">
       <c r="A15" s="40" t="s">
-        <v>218</v>
+        <v>212</v>
       </c>
       <c r="B15" s="41">
         <v>5.0</v>
@@ -3734,7 +3726,7 @@
         <v>7.0</v>
       </c>
       <c r="D15" s="41" t="s">
-        <v>219</v>
+        <v>213</v>
       </c>
       <c r="E15" s="41">
         <v>37.0</v>
@@ -3746,10 +3738,10 @@
         <v>14.0</v>
       </c>
       <c r="H15" s="41" t="s">
-        <v>220</v>
+        <v>214</v>
       </c>
       <c r="I15" s="41" t="s">
-        <v>221</v>
+        <v>215</v>
       </c>
       <c r="J15" s="41" t="s">
         <v>265</v>
@@ -4821,43 +4813,43 @@
       <c r="EU6" s="33"/>
     </row>
     <row r="7" ht="24.75" customHeight="1">
-      <c r="A7" s="23" t="s">
+      <c r="A7" s="34" t="s">
         <v>164</v>
       </c>
-      <c r="B7" s="23">
-        <v>78.0</v>
-      </c>
-      <c r="C7" s="23">
-        <v>98.0</v>
-      </c>
-      <c r="D7" s="23" t="s">
+      <c r="B7" s="35">
+        <v>79.0</v>
+      </c>
+      <c r="C7" s="35">
+        <v>99.0</v>
+      </c>
+      <c r="D7" s="35" t="s">
         <v>165</v>
       </c>
-      <c r="E7" s="23">
+      <c r="E7" s="35">
         <v>20.0</v>
       </c>
-      <c r="F7" s="23">
+      <c r="F7" s="35">
         <v>7.0</v>
       </c>
-      <c r="G7" s="23">
+      <c r="G7" s="35">
         <v>126.0</v>
       </c>
-      <c r="H7" s="23" t="s">
+      <c r="H7" s="35" t="s">
         <v>172</v>
       </c>
-      <c r="I7" s="23" t="s">
+      <c r="I7" s="35" t="s">
         <v>173</v>
       </c>
-      <c r="J7" s="23" t="s">
+      <c r="J7" s="35" t="s">
         <v>106</v>
       </c>
-      <c r="K7" s="23" t="s">
+      <c r="K7" s="35" t="s">
         <v>107</v>
       </c>
-      <c r="L7" s="23" t="s">
+      <c r="L7" s="35" t="s">
         <v>273</v>
       </c>
-      <c r="M7" s="23" t="s">
+      <c r="M7" s="36" t="s">
         <v>274</v>
       </c>
       <c r="N7" s="33"/>
@@ -5000,43 +4992,43 @@
       <c r="EU7" s="33"/>
     </row>
     <row r="8" ht="22.5" customHeight="1">
-      <c r="A8" s="23" t="s">
-        <v>170</v>
-      </c>
-      <c r="B8" s="23">
+      <c r="A8" s="37" t="s">
+        <v>234</v>
+      </c>
+      <c r="B8" s="38">
         <v>40.0</v>
       </c>
-      <c r="C8" s="23">
+      <c r="C8" s="38">
         <v>50.0</v>
       </c>
-      <c r="D8" s="23" t="s">
+      <c r="D8" s="38" t="s">
         <v>171</v>
       </c>
-      <c r="E8" s="23">
+      <c r="E8" s="38">
         <v>21.0</v>
       </c>
-      <c r="F8" s="23">
+      <c r="F8" s="38">
         <v>6.0</v>
       </c>
-      <c r="G8" s="23">
+      <c r="G8" s="38">
         <v>62.0</v>
       </c>
-      <c r="H8" s="23" t="s">
+      <c r="H8" s="38" t="s">
         <v>180</v>
       </c>
-      <c r="I8" s="23" t="s">
+      <c r="I8" s="38" t="s">
         <v>181</v>
       </c>
-      <c r="J8" s="23" t="s">
+      <c r="J8" s="38" t="s">
         <v>275</v>
       </c>
-      <c r="K8" s="23" t="s">
+      <c r="K8" s="38" t="s">
         <v>276</v>
       </c>
-      <c r="L8" s="23" t="s">
+      <c r="L8" s="38" t="s">
         <v>277</v>
       </c>
-      <c r="M8" s="23" t="s">
+      <c r="M8" s="39" t="s">
         <v>278</v>
       </c>
       <c r="N8" s="33"/>
@@ -5179,43 +5171,43 @@
       <c r="EU8" s="33"/>
     </row>
     <row r="9">
-      <c r="A9" s="23" t="s">
+      <c r="A9" s="37" t="s">
         <v>178</v>
       </c>
-      <c r="B9" s="23">
+      <c r="B9" s="38">
         <v>16.0</v>
       </c>
-      <c r="C9" s="23">
+      <c r="C9" s="38">
         <v>20.0</v>
       </c>
-      <c r="D9" s="23" t="s">
+      <c r="D9" s="38" t="s">
         <v>179</v>
       </c>
-      <c r="E9" s="23">
+      <c r="E9" s="38">
         <v>22.0</v>
       </c>
-      <c r="F9" s="23">
+      <c r="F9" s="38">
         <v>5.0</v>
       </c>
-      <c r="G9" s="23">
+      <c r="G9" s="38">
         <v>30.0</v>
       </c>
-      <c r="H9" s="23" t="s">
+      <c r="H9" s="38" t="s">
         <v>206</v>
       </c>
-      <c r="I9" s="23" t="s">
+      <c r="I9" s="38" t="s">
         <v>207</v>
       </c>
-      <c r="J9" s="23" t="s">
+      <c r="J9" s="38" t="s">
         <v>279</v>
       </c>
-      <c r="K9" s="23" t="s">
+      <c r="K9" s="38" t="s">
         <v>280</v>
       </c>
-      <c r="L9" s="23" t="s">
+      <c r="L9" s="38" t="s">
         <v>281</v>
       </c>
-      <c r="M9" s="23" t="s">
+      <c r="M9" s="39" t="s">
         <v>282</v>
       </c>
       <c r="N9" s="33"/>
@@ -5358,43 +5350,43 @@
       <c r="EU9" s="33"/>
     </row>
     <row r="10">
-      <c r="A10" s="23" t="s">
+      <c r="A10" s="37" t="s">
         <v>186</v>
       </c>
-      <c r="B10" s="23">
+      <c r="B10" s="38">
         <v>12.0</v>
       </c>
-      <c r="C10" s="23">
+      <c r="C10" s="38">
         <v>15.0</v>
       </c>
-      <c r="D10" s="23" t="s">
+      <c r="D10" s="38" t="s">
         <v>187</v>
       </c>
-      <c r="E10" s="23">
+      <c r="E10" s="38">
         <v>23.0</v>
       </c>
-      <c r="F10" s="23">
+      <c r="F10" s="38">
         <v>5.0</v>
       </c>
-      <c r="G10" s="23">
+      <c r="G10" s="38">
         <v>30.0</v>
       </c>
-      <c r="H10" s="23" t="s">
+      <c r="H10" s="38" t="s">
         <v>206</v>
       </c>
-      <c r="I10" s="23" t="s">
+      <c r="I10" s="38" t="s">
         <v>207</v>
       </c>
-      <c r="J10" s="23" t="s">
+      <c r="J10" s="38" t="s">
         <v>283</v>
       </c>
-      <c r="K10" s="23" t="s">
+      <c r="K10" s="38" t="s">
         <v>284</v>
       </c>
-      <c r="L10" s="23" t="s">
+      <c r="L10" s="38" t="s">
         <v>285</v>
       </c>
-      <c r="M10" s="23" t="s">
+      <c r="M10" s="39" t="s">
         <v>286</v>
       </c>
       <c r="N10" s="33"/>
@@ -5537,43 +5529,43 @@
       <c r="EU10" s="33"/>
     </row>
     <row r="11">
-      <c r="A11" s="23" t="s">
+      <c r="A11" s="37" t="s">
         <v>192</v>
       </c>
-      <c r="B11" s="23">
+      <c r="B11" s="38">
         <v>11.0</v>
       </c>
-      <c r="C11" s="23">
+      <c r="C11" s="38">
         <v>14.0</v>
       </c>
-      <c r="D11" s="23" t="s">
+      <c r="D11" s="38" t="s">
         <v>193</v>
       </c>
-      <c r="E11" s="23">
+      <c r="E11" s="38">
         <v>24.0</v>
       </c>
-      <c r="F11" s="23">
+      <c r="F11" s="38">
         <v>4.0</v>
       </c>
-      <c r="G11" s="23">
+      <c r="G11" s="38">
         <v>14.0</v>
       </c>
-      <c r="H11" s="23" t="s">
-        <v>220</v>
-      </c>
-      <c r="I11" s="23" t="s">
-        <v>221</v>
-      </c>
-      <c r="J11" s="23" t="s">
+      <c r="H11" s="38" t="s">
+        <v>214</v>
+      </c>
+      <c r="I11" s="38" t="s">
+        <v>215</v>
+      </c>
+      <c r="J11" s="38" t="s">
         <v>287</v>
       </c>
-      <c r="K11" s="23" t="s">
+      <c r="K11" s="38" t="s">
         <v>288</v>
       </c>
-      <c r="L11" s="23" t="s">
+      <c r="L11" s="38" t="s">
         <v>289</v>
       </c>
-      <c r="M11" s="23" t="s">
+      <c r="M11" s="39" t="s">
         <v>290</v>
       </c>
       <c r="N11" s="33"/>
@@ -5716,43 +5708,43 @@
       <c r="EU11" s="33"/>
     </row>
     <row r="12">
-      <c r="A12" s="23" t="s">
-        <v>198</v>
-      </c>
-      <c r="B12" s="23">
+      <c r="A12" s="37" t="s">
+        <v>251</v>
+      </c>
+      <c r="B12" s="38">
         <v>10.0</v>
       </c>
-      <c r="C12" s="23">
+      <c r="C12" s="38">
         <v>13.0</v>
       </c>
-      <c r="D12" s="23" t="s">
+      <c r="D12" s="38" t="s">
         <v>199</v>
       </c>
-      <c r="E12" s="23">
+      <c r="E12" s="38">
         <v>25.0</v>
       </c>
-      <c r="F12" s="23">
+      <c r="F12" s="38">
         <v>4.0</v>
       </c>
-      <c r="G12" s="23">
+      <c r="G12" s="38">
         <v>14.0</v>
       </c>
-      <c r="H12" s="23" t="s">
-        <v>220</v>
-      </c>
-      <c r="I12" s="23" t="s">
-        <v>221</v>
-      </c>
-      <c r="J12" s="23" t="s">
+      <c r="H12" s="38" t="s">
+        <v>214</v>
+      </c>
+      <c r="I12" s="38" t="s">
+        <v>215</v>
+      </c>
+      <c r="J12" s="38" t="s">
         <v>291</v>
       </c>
-      <c r="K12" s="23" t="s">
+      <c r="K12" s="38" t="s">
         <v>292</v>
       </c>
-      <c r="L12" s="23" t="s">
+      <c r="L12" s="38" t="s">
         <v>293</v>
       </c>
-      <c r="M12" s="23" t="s">
+      <c r="M12" s="39" t="s">
         <v>294</v>
       </c>
       <c r="N12" s="33"/>
@@ -5895,44 +5887,44 @@
       <c r="EU12" s="33"/>
     </row>
     <row r="13">
-      <c r="A13" s="23" t="s">
+      <c r="A13" s="37" t="s">
+        <v>256</v>
+      </c>
+      <c r="B13" s="38">
+        <v>9.0</v>
+      </c>
+      <c r="C13" s="38">
+        <v>12.0</v>
+      </c>
+      <c r="D13" s="38" t="s">
+        <v>221</v>
+      </c>
+      <c r="E13" s="38">
+        <v>99.0</v>
+      </c>
+      <c r="F13" s="38">
+        <v>4.0</v>
+      </c>
+      <c r="G13" s="38">
+        <v>14.0</v>
+      </c>
+      <c r="H13" s="38" t="s">
+        <v>214</v>
+      </c>
+      <c r="I13" s="38" t="s">
+        <v>215</v>
+      </c>
+      <c r="J13" s="38" t="s">
         <v>295</v>
       </c>
-      <c r="B13" s="23">
-        <v>10.0</v>
-      </c>
-      <c r="C13" s="23">
-        <v>13.0</v>
-      </c>
-      <c r="D13" s="23" t="s">
-        <v>213</v>
-      </c>
-      <c r="E13" s="23">
-        <v>99.0</v>
-      </c>
-      <c r="F13" s="23">
-        <v>4.0</v>
-      </c>
-      <c r="G13" s="23">
-        <v>14.0</v>
-      </c>
-      <c r="H13" s="23" t="s">
-        <v>220</v>
-      </c>
-      <c r="I13" s="23" t="s">
-        <v>221</v>
-      </c>
-      <c r="J13" s="23" t="s">
+      <c r="K13" s="38" t="s">
         <v>296</v>
       </c>
-      <c r="K13" s="23" t="s">
+      <c r="L13" s="38" t="s">
         <v>297</v>
       </c>
-      <c r="L13" s="23" t="s">
+      <c r="M13" s="39" t="s">
         <v>298</v>
-      </c>
-      <c r="M13" s="23" t="s">
-        <v>299</v>
       </c>
       <c r="N13" s="33"/>
       <c r="O13" s="33"/>
@@ -6074,44 +6066,44 @@
       <c r="EU13" s="33"/>
     </row>
     <row r="14">
-      <c r="A14" s="23" t="s">
+      <c r="A14" s="37" t="s">
         <v>204</v>
       </c>
-      <c r="B14" s="23">
+      <c r="B14" s="38">
         <v>8.0</v>
       </c>
-      <c r="C14" s="23">
+      <c r="C14" s="38">
         <v>10.0</v>
       </c>
-      <c r="D14" s="23" t="s">
+      <c r="D14" s="38" t="s">
         <v>205</v>
       </c>
-      <c r="E14" s="23">
+      <c r="E14" s="38">
         <v>26.0</v>
       </c>
-      <c r="F14" s="23">
+      <c r="F14" s="38">
         <v>4.0</v>
       </c>
-      <c r="G14" s="23">
+      <c r="G14" s="38">
         <v>14.0</v>
       </c>
-      <c r="H14" s="23" t="s">
-        <v>220</v>
-      </c>
-      <c r="I14" s="23" t="s">
-        <v>221</v>
-      </c>
-      <c r="J14" s="23" t="s">
+      <c r="H14" s="38" t="s">
+        <v>214</v>
+      </c>
+      <c r="I14" s="38" t="s">
+        <v>215</v>
+      </c>
+      <c r="J14" s="38" t="s">
+        <v>299</v>
+      </c>
+      <c r="K14" s="38" t="s">
         <v>300</v>
       </c>
-      <c r="K14" s="23" t="s">
+      <c r="L14" s="38" t="s">
         <v>301</v>
       </c>
-      <c r="L14" s="23" t="s">
+      <c r="M14" s="39" t="s">
         <v>302</v>
-      </c>
-      <c r="M14" s="23" t="s">
-        <v>303</v>
       </c>
       <c r="N14" s="33"/>
       <c r="O14" s="33"/>
@@ -6253,44 +6245,44 @@
       <c r="EU14" s="33"/>
     </row>
     <row r="15">
-      <c r="A15" s="23" t="s">
-        <v>218</v>
-      </c>
-      <c r="B15" s="23">
+      <c r="A15" s="40" t="s">
+        <v>212</v>
+      </c>
+      <c r="B15" s="41">
         <v>5.0</v>
       </c>
-      <c r="C15" s="23">
+      <c r="C15" s="41">
         <v>7.0</v>
       </c>
-      <c r="D15" s="23" t="s">
-        <v>219</v>
-      </c>
-      <c r="E15" s="23">
+      <c r="D15" s="41" t="s">
+        <v>213</v>
+      </c>
+      <c r="E15" s="41">
         <v>27.0</v>
       </c>
-      <c r="F15" s="23">
+      <c r="F15" s="41">
         <v>4.0</v>
       </c>
-      <c r="G15" s="23">
+      <c r="G15" s="41">
         <v>14.0</v>
       </c>
-      <c r="H15" s="23" t="s">
-        <v>220</v>
-      </c>
-      <c r="I15" s="23" t="s">
-        <v>221</v>
-      </c>
-      <c r="J15" s="23" t="s">
+      <c r="H15" s="41" t="s">
+        <v>214</v>
+      </c>
+      <c r="I15" s="41" t="s">
+        <v>215</v>
+      </c>
+      <c r="J15" s="41" t="s">
+        <v>303</v>
+      </c>
+      <c r="K15" s="41" t="s">
         <v>304</v>
       </c>
-      <c r="K15" s="23" t="s">
+      <c r="L15" s="41" t="s">
         <v>305</v>
       </c>
-      <c r="L15" s="23" t="s">
+      <c r="M15" s="42" t="s">
         <v>306</v>
-      </c>
-      <c r="M15" s="23" t="s">
-        <v>307</v>
       </c>
       <c r="N15" s="33"/>
       <c r="O15" s="33"/>
@@ -6436,16 +6428,19 @@
         <v>269</v>
       </c>
       <c r="B16" s="43">
-        <v>190.0</v>
+        <f t="shared" ref="B16:C16" si="1">SUM(B7:B15)</f>
+        <v>190</v>
       </c>
       <c r="C16" s="43">
-        <v>240.0</v>
+        <f t="shared" si="1"/>
+        <v>240</v>
       </c>
       <c r="D16" s="44"/>
       <c r="E16" s="44"/>
       <c r="F16" s="44"/>
       <c r="G16" s="43">
-        <v>318.0</v>
+        <f>SUM(G7:G15)</f>
+        <v>318</v>
       </c>
       <c r="H16" s="44"/>
       <c r="I16" s="44"/>
@@ -6750,7 +6745,7 @@
         <v>228</v>
       </c>
       <c r="B18" s="29" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="C18" s="44"/>
       <c r="D18" s="33"/>
@@ -6927,7 +6922,7 @@
         <v>150</v>
       </c>
       <c r="B1" s="29" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
       <c r="C1" s="31"/>
       <c r="D1" s="32"/>
@@ -6965,7 +6960,7 @@
         <v>79</v>
       </c>
       <c r="B3" s="29" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
       <c r="C3" s="44"/>
       <c r="D3" s="33"/>
@@ -7051,371 +7046,371 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="23" t="s">
+      <c r="A7" s="48" t="s">
         <v>164</v>
       </c>
-      <c r="B7" s="23">
-        <v>20.0</v>
-      </c>
-      <c r="C7" s="23">
-        <v>25.0</v>
-      </c>
-      <c r="D7" s="23" t="s">
+      <c r="B7" s="48">
+        <v>15.0</v>
+      </c>
+      <c r="C7" s="48">
+        <v>19.0</v>
+      </c>
+      <c r="D7" s="48" t="s">
         <v>165</v>
       </c>
-      <c r="E7" s="23">
+      <c r="E7" s="48">
         <v>40.0</v>
       </c>
-      <c r="F7" s="23">
+      <c r="F7" s="48">
         <v>5.0</v>
       </c>
-      <c r="G7" s="23">
+      <c r="G7" s="48">
         <v>30.0</v>
       </c>
-      <c r="H7" s="23" t="s">
+      <c r="H7" s="48" t="s">
         <v>206</v>
       </c>
-      <c r="I7" s="23" t="s">
+      <c r="I7" s="48" t="s">
         <v>207</v>
       </c>
-      <c r="J7" s="23" t="s">
+      <c r="J7" s="48" t="s">
         <v>112</v>
       </c>
-      <c r="K7" s="23" t="s">
+      <c r="K7" s="48" t="s">
         <v>113</v>
       </c>
-      <c r="L7" s="23" t="s">
+      <c r="L7" s="48" t="s">
+        <v>310</v>
+      </c>
+      <c r="M7" s="48" t="s">
         <v>311</v>
       </c>
-      <c r="M7" s="23" t="s">
+    </row>
+    <row r="8">
+      <c r="A8" s="48" t="s">
+        <v>170</v>
+      </c>
+      <c r="B8" s="48">
+        <v>13.0</v>
+      </c>
+      <c r="C8" s="48">
+        <v>17.0</v>
+      </c>
+      <c r="D8" s="48" t="s">
+        <v>171</v>
+      </c>
+      <c r="E8" s="48">
+        <v>41.0</v>
+      </c>
+      <c r="F8" s="48">
+        <v>5.0</v>
+      </c>
+      <c r="G8" s="48">
+        <v>30.0</v>
+      </c>
+      <c r="H8" s="48" t="s">
+        <v>206</v>
+      </c>
+      <c r="I8" s="48" t="s">
+        <v>207</v>
+      </c>
+      <c r="J8" s="48" t="s">
         <v>312</v>
       </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="23" t="s">
-        <v>170</v>
-      </c>
-      <c r="B8" s="23">
+      <c r="K8" s="48" t="s">
+        <v>313</v>
+      </c>
+      <c r="L8" s="48" t="s">
+        <v>314</v>
+      </c>
+      <c r="M8" s="48" t="s">
+        <v>315</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="48" t="s">
+        <v>178</v>
+      </c>
+      <c r="B9" s="48">
+        <v>12.0</v>
+      </c>
+      <c r="C9" s="48">
+        <v>15.0</v>
+      </c>
+      <c r="D9" s="48" t="s">
+        <v>179</v>
+      </c>
+      <c r="E9" s="48">
+        <v>42.0</v>
+      </c>
+      <c r="F9" s="48">
+        <v>5.0</v>
+      </c>
+      <c r="G9" s="48">
+        <v>30.0</v>
+      </c>
+      <c r="H9" s="48" t="s">
+        <v>206</v>
+      </c>
+      <c r="I9" s="48" t="s">
+        <v>207</v>
+      </c>
+      <c r="J9" s="48" t="s">
+        <v>316</v>
+      </c>
+      <c r="K9" s="48" t="s">
+        <v>317</v>
+      </c>
+      <c r="L9" s="48" t="s">
+        <v>318</v>
+      </c>
+      <c r="M9" s="48" t="s">
+        <v>319</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="48" t="s">
+        <v>186</v>
+      </c>
+      <c r="B10" s="48">
+        <v>11.0</v>
+      </c>
+      <c r="C10" s="48">
+        <v>14.0</v>
+      </c>
+      <c r="D10" s="48" t="s">
+        <v>187</v>
+      </c>
+      <c r="E10" s="48">
+        <v>43.0</v>
+      </c>
+      <c r="F10" s="48">
+        <v>4.0</v>
+      </c>
+      <c r="G10" s="48">
+        <v>14.0</v>
+      </c>
+      <c r="H10" s="48" t="s">
+        <v>214</v>
+      </c>
+      <c r="I10" s="48" t="s">
+        <v>215</v>
+      </c>
+      <c r="J10" s="48" t="s">
+        <v>320</v>
+      </c>
+      <c r="K10" s="48" t="s">
+        <v>321</v>
+      </c>
+      <c r="L10" s="48" t="s">
+        <v>322</v>
+      </c>
+      <c r="M10" s="48" t="s">
+        <v>323</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="48" t="s">
+        <v>192</v>
+      </c>
+      <c r="B11" s="48">
+        <v>10.0</v>
+      </c>
+      <c r="C11" s="48">
         <v>13.0</v>
       </c>
-      <c r="C8" s="23">
-        <v>17.0</v>
-      </c>
-      <c r="D8" s="23" t="s">
-        <v>171</v>
-      </c>
-      <c r="E8" s="23">
-        <v>41.0</v>
-      </c>
-      <c r="F8" s="23">
-        <v>5.0</v>
-      </c>
-      <c r="G8" s="23">
-        <v>30.0</v>
-      </c>
-      <c r="H8" s="23" t="s">
-        <v>206</v>
-      </c>
-      <c r="I8" s="23" t="s">
-        <v>207</v>
-      </c>
-      <c r="J8" s="23" t="s">
-        <v>313</v>
-      </c>
-      <c r="K8" s="23" t="s">
-        <v>314</v>
-      </c>
-      <c r="L8" s="23" t="s">
-        <v>315</v>
-      </c>
-      <c r="M8" s="23" t="s">
-        <v>316</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="23" t="s">
-        <v>178</v>
-      </c>
-      <c r="B9" s="23">
+      <c r="D11" s="48" t="s">
+        <v>193</v>
+      </c>
+      <c r="E11" s="48">
+        <v>44.0</v>
+      </c>
+      <c r="F11" s="48">
+        <v>4.0</v>
+      </c>
+      <c r="G11" s="48">
+        <v>14.0</v>
+      </c>
+      <c r="H11" s="48" t="s">
+        <v>214</v>
+      </c>
+      <c r="I11" s="48" t="s">
+        <v>215</v>
+      </c>
+      <c r="J11" s="48" t="s">
+        <v>324</v>
+      </c>
+      <c r="K11" s="48" t="s">
+        <v>325</v>
+      </c>
+      <c r="L11" s="48" t="s">
+        <v>326</v>
+      </c>
+      <c r="M11" s="48" t="s">
+        <v>327</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="48" t="s">
+        <v>198</v>
+      </c>
+      <c r="B12" s="48">
+        <v>10.0</v>
+      </c>
+      <c r="C12" s="48">
+        <v>13.0</v>
+      </c>
+      <c r="D12" s="48" t="s">
+        <v>199</v>
+      </c>
+      <c r="E12" s="48">
+        <v>45.0</v>
+      </c>
+      <c r="F12" s="48">
+        <v>4.0</v>
+      </c>
+      <c r="G12" s="48">
+        <v>14.0</v>
+      </c>
+      <c r="H12" s="48" t="s">
+        <v>214</v>
+      </c>
+      <c r="I12" s="48" t="s">
+        <v>215</v>
+      </c>
+      <c r="J12" s="48" t="s">
+        <v>328</v>
+      </c>
+      <c r="K12" s="48" t="s">
+        <v>329</v>
+      </c>
+      <c r="L12" s="48" t="s">
+        <v>330</v>
+      </c>
+      <c r="M12" s="48" t="s">
+        <v>331</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="48" t="s">
+        <v>204</v>
+      </c>
+      <c r="B13" s="48">
+        <v>10.0</v>
+      </c>
+      <c r="C13" s="48">
+        <v>13.0</v>
+      </c>
+      <c r="D13" s="48" t="s">
+        <v>205</v>
+      </c>
+      <c r="E13" s="48">
+        <v>46.0</v>
+      </c>
+      <c r="F13" s="48">
+        <v>4.0</v>
+      </c>
+      <c r="G13" s="48">
+        <v>14.0</v>
+      </c>
+      <c r="H13" s="48" t="s">
+        <v>214</v>
+      </c>
+      <c r="I13" s="48" t="s">
+        <v>215</v>
+      </c>
+      <c r="J13" s="48" t="s">
+        <v>332</v>
+      </c>
+      <c r="K13" s="48" t="s">
+        <v>333</v>
+      </c>
+      <c r="L13" s="48" t="s">
+        <v>334</v>
+      </c>
+      <c r="M13" s="48" t="s">
+        <v>335</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="48" t="s">
+        <v>336</v>
+      </c>
+      <c r="B14" s="48">
+        <v>9.0</v>
+      </c>
+      <c r="C14" s="48">
         <v>12.0</v>
       </c>
-      <c r="C9" s="23">
-        <v>15.0</v>
-      </c>
-      <c r="D9" s="23" t="s">
-        <v>179</v>
-      </c>
-      <c r="E9" s="23">
-        <v>42.0</v>
-      </c>
-      <c r="F9" s="23">
-        <v>5.0</v>
-      </c>
-      <c r="G9" s="23">
-        <v>30.0</v>
-      </c>
-      <c r="H9" s="23" t="s">
-        <v>206</v>
-      </c>
-      <c r="I9" s="23" t="s">
-        <v>207</v>
-      </c>
-      <c r="J9" s="23" t="s">
-        <v>317</v>
-      </c>
-      <c r="K9" s="23" t="s">
-        <v>318</v>
-      </c>
-      <c r="L9" s="23" t="s">
-        <v>319</v>
-      </c>
-      <c r="M9" s="23" t="s">
-        <v>320</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="23" t="s">
-        <v>186</v>
-      </c>
-      <c r="B10" s="23">
-        <v>11.0</v>
-      </c>
-      <c r="C10" s="23">
+      <c r="D14" s="48" t="s">
+        <v>221</v>
+      </c>
+      <c r="E14" s="48">
+        <v>99.0</v>
+      </c>
+      <c r="F14" s="48">
+        <v>4.0</v>
+      </c>
+      <c r="G14" s="48">
         <v>14.0</v>
       </c>
-      <c r="D10" s="23" t="s">
-        <v>187</v>
-      </c>
-      <c r="E10" s="23">
-        <v>43.0</v>
-      </c>
-      <c r="F10" s="23">
+      <c r="H14" s="48" t="s">
+        <v>214</v>
+      </c>
+      <c r="I14" s="48" t="s">
+        <v>215</v>
+      </c>
+      <c r="J14" s="48" t="s">
+        <v>337</v>
+      </c>
+      <c r="K14" s="48" t="s">
+        <v>338</v>
+      </c>
+      <c r="L14" s="48" t="s">
+        <v>339</v>
+      </c>
+      <c r="M14" s="48" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="48" t="s">
+        <v>212</v>
+      </c>
+      <c r="B15" s="48">
+        <v>6.0</v>
+      </c>
+      <c r="C15" s="48">
+        <v>8.0</v>
+      </c>
+      <c r="D15" s="48" t="s">
+        <v>213</v>
+      </c>
+      <c r="E15" s="48">
+        <v>47.0</v>
+      </c>
+      <c r="F15" s="48">
         <v>4.0</v>
       </c>
-      <c r="G10" s="23">
+      <c r="G15" s="48">
         <v>14.0</v>
       </c>
-      <c r="H10" s="23" t="s">
-        <v>220</v>
-      </c>
-      <c r="I10" s="23" t="s">
-        <v>221</v>
-      </c>
-      <c r="J10" s="23" t="s">
-        <v>321</v>
-      </c>
-      <c r="K10" s="23" t="s">
-        <v>322</v>
-      </c>
-      <c r="L10" s="23" t="s">
-        <v>323</v>
-      </c>
-      <c r="M10" s="23" t="s">
-        <v>324</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="23" t="s">
-        <v>192</v>
-      </c>
-      <c r="B11" s="23">
-        <v>10.0</v>
-      </c>
-      <c r="C11" s="23">
-        <v>13.0</v>
-      </c>
-      <c r="D11" s="23" t="s">
-        <v>193</v>
-      </c>
-      <c r="E11" s="23">
-        <v>44.0</v>
-      </c>
-      <c r="F11" s="23">
-        <v>4.0</v>
-      </c>
-      <c r="G11" s="23">
-        <v>14.0</v>
-      </c>
-      <c r="H11" s="23" t="s">
-        <v>220</v>
-      </c>
-      <c r="I11" s="23" t="s">
-        <v>221</v>
-      </c>
-      <c r="J11" s="23" t="s">
-        <v>325</v>
-      </c>
-      <c r="K11" s="23" t="s">
-        <v>326</v>
-      </c>
-      <c r="L11" s="23" t="s">
-        <v>327</v>
-      </c>
-      <c r="M11" s="23" t="s">
-        <v>328</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="23" t="s">
-        <v>198</v>
-      </c>
-      <c r="B12" s="23">
-        <v>9.0</v>
-      </c>
-      <c r="C12" s="23">
-        <v>12.0</v>
-      </c>
-      <c r="D12" s="23" t="s">
-        <v>199</v>
-      </c>
-      <c r="E12" s="23">
-        <v>45.0</v>
-      </c>
-      <c r="F12" s="23">
-        <v>4.0</v>
-      </c>
-      <c r="G12" s="23">
-        <v>14.0</v>
-      </c>
-      <c r="H12" s="23" t="s">
-        <v>220</v>
-      </c>
-      <c r="I12" s="23" t="s">
-        <v>221</v>
-      </c>
-      <c r="J12" s="23" t="s">
-        <v>329</v>
-      </c>
-      <c r="K12" s="23" t="s">
-        <v>330</v>
-      </c>
-      <c r="L12" s="23" t="s">
-        <v>331</v>
-      </c>
-      <c r="M12" s="23" t="s">
-        <v>332</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="23" t="s">
-        <v>204</v>
-      </c>
-      <c r="B13" s="23">
-        <v>8.0</v>
-      </c>
-      <c r="C13" s="23">
-        <v>10.0</v>
-      </c>
-      <c r="D13" s="23" t="s">
-        <v>205</v>
-      </c>
-      <c r="E13" s="23">
-        <v>46.0</v>
-      </c>
-      <c r="F13" s="23">
-        <v>4.0</v>
-      </c>
-      <c r="G13" s="23">
-        <v>14.0</v>
-      </c>
-      <c r="H13" s="23" t="s">
-        <v>220</v>
-      </c>
-      <c r="I13" s="23" t="s">
-        <v>221</v>
-      </c>
-      <c r="J13" s="23" t="s">
-        <v>333</v>
-      </c>
-      <c r="K13" s="23" t="s">
-        <v>334</v>
-      </c>
-      <c r="L13" s="23" t="s">
-        <v>335</v>
-      </c>
-      <c r="M13" s="23" t="s">
-        <v>336</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="23" t="s">
-        <v>295</v>
-      </c>
-      <c r="B14" s="23">
-        <v>7.0</v>
-      </c>
-      <c r="C14" s="23">
-        <v>9.0</v>
-      </c>
-      <c r="D14" s="23" t="s">
-        <v>213</v>
-      </c>
-      <c r="E14" s="23">
-        <v>99.0</v>
-      </c>
-      <c r="F14" s="23">
-        <v>4.0</v>
-      </c>
-      <c r="G14" s="23">
-        <v>14.0</v>
-      </c>
-      <c r="H14" s="23" t="s">
-        <v>220</v>
-      </c>
-      <c r="I14" s="23" t="s">
-        <v>221</v>
-      </c>
-      <c r="J14" s="23" t="s">
-        <v>337</v>
-      </c>
-      <c r="K14" s="23" t="s">
-        <v>338</v>
-      </c>
-      <c r="L14" s="23" t="s">
-        <v>339</v>
-      </c>
-      <c r="M14" s="23" t="s">
-        <v>340</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="23" t="s">
-        <v>218</v>
-      </c>
-      <c r="B15" s="23">
-        <v>6.0</v>
-      </c>
-      <c r="C15" s="23">
-        <v>8.0</v>
-      </c>
-      <c r="D15" s="23" t="s">
-        <v>219</v>
-      </c>
-      <c r="E15" s="23">
-        <v>47.0</v>
-      </c>
-      <c r="F15" s="23">
-        <v>4.0</v>
-      </c>
-      <c r="G15" s="23">
-        <v>14.0</v>
-      </c>
-      <c r="H15" s="23" t="s">
-        <v>220</v>
-      </c>
-      <c r="I15" s="23" t="s">
-        <v>221</v>
-      </c>
-      <c r="J15" s="23" t="s">
+      <c r="H15" s="48" t="s">
+        <v>214</v>
+      </c>
+      <c r="I15" s="48" t="s">
+        <v>215</v>
+      </c>
+      <c r="J15" s="48" t="s">
         <v>341</v>
       </c>
-      <c r="K15" s="23" t="s">
+      <c r="K15" s="48" t="s">
         <v>342</v>
       </c>
-      <c r="L15" s="23" t="s">
+      <c r="L15" s="48" t="s">
         <v>343</v>
       </c>
-      <c r="M15" s="23" t="s">
+      <c r="M15" s="48" t="s">
         <v>344</v>
       </c>
     </row>
@@ -7424,17 +7419,17 @@
         <v>269</v>
       </c>
       <c r="B16" s="43">
-        <v>96.0</v>
+        <f t="shared" ref="B16:C16" si="1">SUM(B7:B15)</f>
+        <v>96</v>
       </c>
       <c r="C16" s="43">
-        <v>123.0</v>
+        <f t="shared" si="1"/>
+        <v>124</v>
       </c>
       <c r="D16" s="33"/>
       <c r="E16" s="33"/>
       <c r="F16" s="33"/>
-      <c r="G16" s="43">
-        <v>174.0</v>
-      </c>
+      <c r="G16" s="43"/>
       <c r="H16" s="33"/>
       <c r="I16" s="33"/>
       <c r="J16" s="33"/>
@@ -7461,7 +7456,7 @@
       <c r="A18" s="25" t="s">
         <v>228</v>
       </c>
-      <c r="B18" s="48" t="s">
+      <c r="B18" s="49" t="s">
         <v>345</v>
       </c>
       <c r="C18" s="27"/>
@@ -7608,43 +7603,43 @@
       <c r="N5" s="33"/>
     </row>
     <row r="6">
-      <c r="A6" s="22" t="s">
+      <c r="A6" s="50" t="s">
         <v>155</v>
       </c>
-      <c r="B6" s="22" t="s">
+      <c r="B6" s="50" t="s">
         <v>156</v>
       </c>
-      <c r="C6" s="22" t="s">
+      <c r="C6" s="50" t="s">
         <v>157</v>
       </c>
-      <c r="D6" s="22" t="s">
+      <c r="D6" s="50" t="s">
         <v>158</v>
       </c>
-      <c r="E6" s="49" t="s">
+      <c r="E6" s="50" t="s">
         <v>159</v>
       </c>
-      <c r="F6" s="22" t="s">
+      <c r="F6" s="50" t="s">
         <v>160</v>
       </c>
-      <c r="G6" s="22" t="s">
+      <c r="G6" s="50" t="s">
         <v>161</v>
       </c>
-      <c r="H6" s="22" t="s">
+      <c r="H6" s="50" t="s">
         <v>14</v>
       </c>
-      <c r="I6" s="22" t="s">
+      <c r="I6" s="50" t="s">
         <v>162</v>
       </c>
-      <c r="J6" s="22" t="s">
+      <c r="J6" s="50" t="s">
         <v>127</v>
       </c>
-      <c r="K6" s="22" t="s">
+      <c r="K6" s="50" t="s">
         <v>15</v>
       </c>
-      <c r="L6" s="22" t="s">
+      <c r="L6" s="50" t="s">
         <v>16</v>
       </c>
-      <c r="M6" s="22" t="s">
+      <c r="M6" s="50" t="s">
         <v>163</v>
       </c>
       <c r="N6" s="33"/>
@@ -7654,15 +7649,15 @@
         <v>164</v>
       </c>
       <c r="B7" s="35">
-        <v>32.0</v>
+        <v>31.0</v>
       </c>
       <c r="C7" s="35">
-        <v>40.0</v>
+        <v>39.0</v>
       </c>
       <c r="D7" s="35" t="s">
         <v>165</v>
       </c>
-      <c r="E7" s="50">
+      <c r="E7" s="35">
         <v>50.0</v>
       </c>
       <c r="F7" s="35">
@@ -7704,7 +7699,7 @@
       <c r="D8" s="38" t="s">
         <v>171</v>
       </c>
-      <c r="E8" s="51">
+      <c r="E8" s="38">
         <v>51.0</v>
       </c>
       <c r="F8" s="38">
@@ -7746,7 +7741,7 @@
       <c r="D9" s="38" t="s">
         <v>179</v>
       </c>
-      <c r="E9" s="51">
+      <c r="E9" s="38">
         <v>52.0</v>
       </c>
       <c r="F9" s="38">
@@ -7756,10 +7751,10 @@
         <v>14.0</v>
       </c>
       <c r="H9" s="38" t="s">
-        <v>220</v>
+        <v>214</v>
       </c>
       <c r="I9" s="38" t="s">
-        <v>221</v>
+        <v>215</v>
       </c>
       <c r="J9" s="38" t="s">
         <v>354</v>
@@ -7788,7 +7783,7 @@
       <c r="D10" s="38" t="s">
         <v>187</v>
       </c>
-      <c r="E10" s="51">
+      <c r="E10" s="38">
         <v>53.0</v>
       </c>
       <c r="F10" s="38">
@@ -7798,10 +7793,10 @@
         <v>14.0</v>
       </c>
       <c r="H10" s="38" t="s">
-        <v>220</v>
+        <v>214</v>
       </c>
       <c r="I10" s="38" t="s">
-        <v>221</v>
+        <v>215</v>
       </c>
       <c r="J10" s="38" t="s">
         <v>358</v>
@@ -7819,19 +7814,19 @@
     </row>
     <row r="11">
       <c r="A11" s="37" t="s">
-        <v>192</v>
+        <v>256</v>
       </c>
       <c r="B11" s="38">
-        <v>8.0</v>
+        <v>9.0</v>
       </c>
       <c r="C11" s="38">
-        <v>10.0</v>
+        <v>12.0</v>
       </c>
       <c r="D11" s="38" t="s">
-        <v>193</v>
-      </c>
-      <c r="E11" s="51">
-        <v>54.0</v>
+        <v>221</v>
+      </c>
+      <c r="E11" s="38">
+        <v>55.0</v>
       </c>
       <c r="F11" s="38">
         <v>4.0</v>
@@ -7840,10 +7835,10 @@
         <v>14.0</v>
       </c>
       <c r="H11" s="38" t="s">
-        <v>220</v>
+        <v>214</v>
       </c>
       <c r="I11" s="38" t="s">
-        <v>221</v>
+        <v>215</v>
       </c>
       <c r="J11" s="38" t="s">
         <v>362</v>
@@ -7861,7 +7856,7 @@
     </row>
     <row r="12">
       <c r="A12" s="37" t="s">
-        <v>256</v>
+        <v>192</v>
       </c>
       <c r="B12" s="38">
         <v>8.0</v>
@@ -7870,10 +7865,10 @@
         <v>10.0</v>
       </c>
       <c r="D12" s="38" t="s">
-        <v>213</v>
-      </c>
-      <c r="E12" s="51">
-        <v>55.0</v>
+        <v>193</v>
+      </c>
+      <c r="E12" s="38">
+        <v>54.0</v>
       </c>
       <c r="F12" s="38">
         <v>4.0</v>
@@ -7882,10 +7877,10 @@
         <v>14.0</v>
       </c>
       <c r="H12" s="38" t="s">
-        <v>220</v>
+        <v>214</v>
       </c>
       <c r="I12" s="38" t="s">
-        <v>221</v>
+        <v>215</v>
       </c>
       <c r="J12" s="38" t="s">
         <v>366</v>
@@ -7914,7 +7909,7 @@
       <c r="D13" s="38" t="s">
         <v>199</v>
       </c>
-      <c r="E13" s="51">
+      <c r="E13" s="38">
         <v>56.0</v>
       </c>
       <c r="F13" s="38">
@@ -7924,10 +7919,10 @@
         <v>14.0</v>
       </c>
       <c r="H13" s="38" t="s">
-        <v>220</v>
+        <v>214</v>
       </c>
       <c r="I13" s="38" t="s">
-        <v>221</v>
+        <v>215</v>
       </c>
       <c r="J13" s="38" t="s">
         <v>370</v>
@@ -7956,7 +7951,7 @@
       <c r="D14" s="38" t="s">
         <v>205</v>
       </c>
-      <c r="E14" s="51">
+      <c r="E14" s="38">
         <v>57.0</v>
       </c>
       <c r="F14" s="38">
@@ -7966,10 +7961,10 @@
         <v>14.0</v>
       </c>
       <c r="H14" s="38" t="s">
-        <v>220</v>
+        <v>214</v>
       </c>
       <c r="I14" s="38" t="s">
-        <v>221</v>
+        <v>215</v>
       </c>
       <c r="J14" s="38" t="s">
         <v>374</v>
@@ -7987,7 +7982,7 @@
     </row>
     <row r="15">
       <c r="A15" s="40" t="s">
-        <v>218</v>
+        <v>212</v>
       </c>
       <c r="B15" s="41">
         <v>5.0</v>
@@ -7996,9 +7991,9 @@
         <v>7.0</v>
       </c>
       <c r="D15" s="41" t="s">
-        <v>219</v>
-      </c>
-      <c r="E15" s="52">
+        <v>213</v>
+      </c>
+      <c r="E15" s="41">
         <v>58.0</v>
       </c>
       <c r="F15" s="41">
@@ -8008,10 +8003,10 @@
         <v>14.0</v>
       </c>
       <c r="H15" s="41" t="s">
-        <v>220</v>
+        <v>214</v>
       </c>
       <c r="I15" s="41" t="s">
-        <v>221</v>
+        <v>215</v>
       </c>
       <c r="J15" s="41" t="s">
         <v>378</v>
@@ -8028,21 +8023,21 @@
       <c r="N15" s="33"/>
     </row>
     <row r="16">
-      <c r="A16" s="25" t="s">
+      <c r="A16" s="51" t="s">
         <v>269</v>
       </c>
-      <c r="B16" s="43">
+      <c r="B16" s="52">
         <f t="shared" ref="B16:C16" si="1">SUM(B7:B15)</f>
         <v>105</v>
       </c>
-      <c r="C16" s="43">
+      <c r="C16" s="52">
         <f t="shared" si="1"/>
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="D16" s="33"/>
       <c r="E16" s="33"/>
       <c r="F16" s="33"/>
-      <c r="G16" s="43">
+      <c r="G16" s="52">
         <f>SUM(G7:G15)</f>
         <v>190</v>
       </c>

</xml_diff>